<commit_message>
📈 Daily Screener Report — 19-May-2026 12:02 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -816,13 +816,13 @@
         <v>0.59</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>139854</v>
+        <v>137942</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.590015</v>
+        <v>51.87985</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.749046</v>
+        <v>37.232964</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -837,7 +837,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.6461735</v>
+        <v>11.486955</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -950,13 +950,13 @@
         <v>1.14</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>183213</v>
+        <v>183492</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>73.70247999999999</v>
+        <v>73.81461</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>59.035583</v>
+        <v>59.1254</v>
       </c>
       <c r="AD3" s="4" t="inlineStr"/>
       <c r="AE3" s="4" t="n">
@@ -969,7 +969,7 @@
         <v>-1</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>11.879639</v>
+        <v>11.897712</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>44</v>
@@ -1080,13 +1080,13 @@
         <v>0.73</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>411487</v>
+        <v>406142</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>30.645163</v>
+        <v>30.247084</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>23.027498</v>
+        <v>22.728373</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>15.59</v>
@@ -1101,7 +1101,7 @@
         <v>3.6</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>4.280397</v>
+        <v>4.2247953</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>42</v>
@@ -1214,13 +1214,13 @@
         <v>1.55</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>315135</v>
+        <v>313670</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>14.140839</v>
+        <v>14.081297</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>17.93597</v>
+        <v>17.852625</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>27.26</v>
@@ -1235,7 +1235,7 @@
         <v>991.8</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>3.149806</v>
+        <v>3.1351693</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>55</v>
@@ -1348,13 +1348,13 @@
         <v>4.31</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>12643</v>
+        <v>12734</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>30.567175</v>
+        <v>30.785805</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>18.259304</v>
+        <v>18.389902</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>10.66</v>
@@ -1369,7 +1369,7 @@
         <v>5.9</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>3.2903805</v>
+        <v>3.3139148</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>79</v>
@@ -1482,13 +1482,13 @@
         <v>0.82</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>107778</v>
+        <v>107740</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>61.20309</v>
+        <v>61.181015</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>44.07573</v>
+        <v>44.059834</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>41.39</v>
@@ -1503,7 +1503,7 @@
         <v>14.5</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>25.410913</v>
+        <v>25.401749</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>48</v>
@@ -1616,13 +1616,13 @@
         <v>0.73</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>277446</v>
+        <v>276019</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>79.141914</v>
+        <v>78.73487</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>60.736362</v>
+        <v>60.42398</v>
       </c>
       <c r="AD8" s="2" t="n">
         <v>76.34</v>
@@ -1637,7 +1637,7 @@
         <v>27.4</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>53.800995</v>
+        <v>53.52429</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>84</v>
@@ -1750,13 +1750,13 @@
         <v>1.84</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>29439</v>
+        <v>29617</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>26.740614</v>
+        <v>26.902729</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>10.671962</v>
+        <v>10.736661</v>
       </c>
       <c r="AD9" s="4" t="n">
         <v>6.97</v>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="AG9" s="4" t="inlineStr"/>
       <c r="AH9" s="4" t="n">
-        <v>1.634505</v>
+        <v>1.6444142</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>65</v>
@@ -1882,13 +1882,13 @@
         <v>0.6</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>372628</v>
+        <v>373005</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>9.798214</v>
+        <v>9.808138</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>6.994827</v>
+        <v>7.001911</v>
       </c>
       <c r="AD10" s="2" t="inlineStr"/>
       <c r="AE10" s="2" t="n">
@@ -1901,7 +1901,7 @@
         <v>16.2</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>1.0123416</v>
+        <v>1.0133669</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>622</v>
@@ -2012,13 +2012,13 @@
         <v>0.96</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>8943</v>
+        <v>9061</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>79.70238500000001</v>
+        <v>80.46856</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>40.999268</v>
+        <v>41.54123</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -2031,7 +2031,7 @@
         <v>35.8</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>13.719543</v>
+        <v>13.900899</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>0</v>
@@ -2142,13 +2142,13 @@
         <v>1.16</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>151502</v>
+        <v>150950</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>66.59327</v>
+        <v>66.35079</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>69.11971</v>
+        <v>68.86803</v>
       </c>
       <c r="AD12" s="2" t="inlineStr"/>
       <c r="AE12" s="2" t="n">
@@ -2161,10 +2161,10 @@
         <v>26.1</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>17.943857</v>
+        <v>17.878517</v>
       </c>
       <c r="AI12" s="2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AJ12" s="2" t="inlineStr"/>
       <c r="AK12" s="2" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="AB13" s="4" t="inlineStr"/>
       <c r="AC13" s="4" t="n">
-        <v>27.849463</v>
+        <v>27.844086</v>
       </c>
       <c r="AD13" s="4" t="n">
         <v>-2.82</v>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="AG13" s="4" t="inlineStr"/>
       <c r="AH13" s="4" t="n">
-        <v>5.671657</v>
+        <v>5.6705623</v>
       </c>
       <c r="AI13" s="4" t="n">
         <v>0</v>
@@ -2402,13 +2402,13 @@
         <v>0.67</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>376146</v>
+        <v>373582</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>37.22795</v>
+        <v>36.97422</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>48.402573</v>
+        <v>48.07268</v>
       </c>
       <c r="AD14" s="2" t="n">
         <v>13.66</v>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="AG14" s="2" t="inlineStr"/>
       <c r="AH14" s="2" t="n">
-        <v>4.3759727</v>
+        <v>4.346148</v>
       </c>
       <c r="AI14" s="2" t="n">
         <v>5</v>
@@ -2534,13 +2534,13 @@
         <v>0.64</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>453762</v>
+        <v>451627</v>
       </c>
       <c r="AB15" s="4" t="n">
-        <v>41.51921</v>
+        <v>41.323822</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>33.42379</v>
+        <v>33.2665</v>
       </c>
       <c r="AD15" s="4" t="inlineStr"/>
       <c r="AE15" s="4" t="n">
@@ -2553,7 +2553,7 @@
         <v>15.7</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>5.8287253</v>
+        <v>5.8012958</v>
       </c>
       <c r="AI15" s="4" t="n">
         <v>87</v>
@@ -2664,13 +2664,13 @@
         <v>0.7</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>281575</v>
+        <v>281606</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>9.054697000000001</v>
+        <v>9.055688</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>7.9895134</v>
+        <v>7.990388</v>
       </c>
       <c r="AD16" s="2" t="n">
         <v>28.12</v>
@@ -2685,7 +2685,7 @@
         <v>12.9</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>2.363928</v>
+        <v>2.3641868</v>
       </c>
       <c r="AI16" s="2" t="n">
         <v>476</v>
@@ -2798,13 +2798,13 @@
         <v>0.85</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>116099</v>
+        <v>115402</v>
       </c>
       <c r="AB17" s="4" t="n">
-        <v>64.53404</v>
+        <v>64.146416</v>
       </c>
       <c r="AC17" s="4" t="n">
-        <v>48.52542</v>
+        <v>48.233948</v>
       </c>
       <c r="AD17" s="4" t="inlineStr"/>
       <c r="AE17" s="4" t="n">
@@ -2817,7 +2817,7 @@
         <v>35</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>12.766956</v>
+        <v>12.690271</v>
       </c>
       <c r="AI17" s="4" t="n">
         <v>25</v>
@@ -2928,13 +2928,13 @@
         <v>1.29</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>78174</v>
+        <v>77730</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>557.1428</v>
+        <v>553.9796</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>176.0132</v>
+        <v>175.01387</v>
       </c>
       <c r="AD18" s="2" t="inlineStr"/>
       <c r="AE18" s="2" t="n">
@@ -2947,7 +2947,7 @@
         <v>144.4</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>56.439945</v>
+        <v>56.1195</v>
       </c>
       <c r="AI18" s="2" t="n">
         <v>0</v>
@@ -3058,13 +3058,13 @@
         <v>0.76</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>87452</v>
+        <v>87043</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>25.323225</v>
+        <v>25.204933</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>19.88931</v>
+        <v>19.796402</v>
       </c>
       <c r="AD19" s="4" t="inlineStr"/>
       <c r="AE19" s="4" t="n">
@@ -3077,10 +3077,10 @@
         <v>7.6</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>2.5189137</v>
+        <v>2.507147</v>
       </c>
       <c r="AI19" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AJ19" s="4" t="inlineStr"/>
       <c r="AK19" s="4" t="inlineStr">
@@ -3188,13 +3188,13 @@
         <v>1.43</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>1168405</v>
+        <v>1165603</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>43.219917</v>
+        <v>43.11627</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>22.989098</v>
+        <v>22.933964</v>
       </c>
       <c r="AD20" s="2" t="n">
         <v>19.36</v>
@@ -3209,7 +3209,7 @@
         <v>-34</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>7.5228457</v>
+        <v>7.5048046</v>
       </c>
       <c r="AI20" s="2" t="n">
         <v>83</v>
@@ -3322,13 +3322,13 @@
         <v>0.62</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>21378</v>
+        <v>21144</v>
       </c>
       <c r="AB21" s="4" t="n">
-        <v>388.05554</v>
+        <v>383.80554</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>26.865385</v>
+        <v>26.571154</v>
       </c>
       <c r="AD21" s="4" t="n">
         <v>7.27</v>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="AG21" s="4" t="inlineStr"/>
       <c r="AH21" s="4" t="n">
-        <v>4.311728</v>
+        <v>4.264506</v>
       </c>
       <c r="AI21" s="4" t="n">
         <v>7</v>
@@ -3454,13 +3454,13 @@
         <v>2.71</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>263306</v>
+        <v>261023</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>28.762941</v>
+        <v>28.513622</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>11.229788</v>
+        <v>11.132447</v>
       </c>
       <c r="AD22" s="2" t="n">
         <v>11.16</v>
@@ -3475,10 +3475,10 @@
         <v>125.4</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>2.7698402</v>
+        <v>2.745831</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>166</v>
+        <v>191</v>
       </c>
       <c r="AJ22" s="2" t="n">
         <v>0.748</v>
@@ -3588,13 +3588,13 @@
         <v>0.71</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>20411</v>
+        <v>20024</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>23.397161</v>
+        <v>22.9539</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>17.383423</v>
+        <v>17.054092</v>
       </c>
       <c r="AD23" s="4" t="inlineStr"/>
       <c r="AE23" s="4" t="inlineStr"/>
@@ -3605,7 +3605,7 @@
         <v>367.9</v>
       </c>
       <c r="AH23" s="4" t="n">
-        <v>1.2192732</v>
+        <v>1.1961739</v>
       </c>
       <c r="AI23" s="4" t="n">
         <v>33</v>
@@ -3716,13 +3716,13 @@
         <v>0.58</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>18659</v>
+        <v>18957</v>
       </c>
       <c r="AB24" s="2" t="n">
-        <v>57.384483</v>
+        <v>58.30273</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>34.052444</v>
+        <v>34.59734</v>
       </c>
       <c r="AD24" s="2" t="n">
         <v>14.14</v>
@@ -3737,7 +3737,7 @@
         <v>43.7</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>6.4218326</v>
+        <v>6.524593</v>
       </c>
       <c r="AI24" s="2" t="n">
         <v>15</v>
@@ -3850,13 +3850,13 @@
         <v>0.42</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>30920</v>
+        <v>30804</v>
       </c>
       <c r="AB25" s="4" t="n">
-        <v>25.287218</v>
+        <v>25.192358</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>8.876007</v>
+        <v>8.842710500000001</v>
       </c>
       <c r="AD25" s="4" t="n">
         <v>4.88</v>
@@ -3869,7 +3869,7 @@
         <v>68</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>1.2073802</v>
+        <v>1.2028509</v>
       </c>
       <c r="AI25" s="4" t="n">
         <v>79</v>
@@ -3980,13 +3980,13 @@
         <v>0.73</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>23999</v>
+        <v>24001</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>15.580895</v>
+        <v>15.581756</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>12.651418</v>
+        <v>12.652116</v>
       </c>
       <c r="AD26" s="2" t="n">
         <v>12.55</v>
@@ -4001,7 +4001,7 @@
         <v>17.8</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>1.8858393</v>
+        <v>1.8859434</v>
       </c>
       <c r="AI26" s="2" t="n">
         <v>340</v>
@@ -4114,13 +4114,13 @@
         <v>0.52</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>59571</v>
+        <v>59198</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>52.94301</v>
+        <v>52.6114</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>40.231575</v>
+        <v>39.979588</v>
       </c>
       <c r="AD27" s="4" t="n">
         <v>17.23</v>
@@ -4135,7 +4135,7 @@
         <v>27.7</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>8.616531</v>
+        <v>8.562563000000001</v>
       </c>
       <c r="AI27" s="4" t="n">
         <v>72</v>
@@ -4248,13 +4248,13 @@
         <v>0.58</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>110535</v>
+        <v>111168</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>26.383148</v>
+        <v>26.53418</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>20.688011</v>
+        <v>20.806442</v>
       </c>
       <c r="AD28" s="2" t="n">
         <v>11.83</v>
@@ -4269,7 +4269,7 @@
         <v>-86.2</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>2.9354148</v>
+        <v>2.9522188</v>
       </c>
       <c r="AI28" s="2" t="n">
         <v>60</v>
@@ -4382,13 +4382,13 @@
         <v>0.6</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>148941</v>
+        <v>148168</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>60.797676</v>
+        <v>60.48193</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>48.274868</v>
+        <v>48.02416</v>
       </c>
       <c r="AD29" s="4" t="n">
         <v>23.52</v>
@@ -4403,10 +4403,10 @@
         <v>37</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>15.5933</v>
+        <v>15.512319</v>
       </c>
       <c r="AI29" s="4" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>2.38</v>
@@ -4516,13 +4516,13 @@
         <v>1.7</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>277391</v>
+        <v>277716</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>14.83093</v>
+        <v>14.848334</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>14.820517</v>
+        <v>14.979996</v>
       </c>
       <c r="AD30" s="2" t="n">
         <v>16.49</v>
@@ -4537,7 +4537,7 @@
         <v>9.6</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>2.7996547</v>
+        <v>2.8029401</v>
       </c>
       <c r="AI30" s="2" t="n">
         <v>413</v>
@@ -4650,13 +4650,13 @@
         <v>0.89</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>114506</v>
+        <v>113884</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>29.49438</v>
+        <v>29.334166</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>22.376104</v>
+        <v>22.254555</v>
       </c>
       <c r="AD31" s="4" t="n">
         <v>11.74</v>
@@ -4671,7 +4671,7 @@
         <v>-54.6</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>3.478263</v>
+        <v>3.4593687</v>
       </c>
       <c r="AI31" s="4" t="n">
         <v>91</v>
@@ -4784,13 +4784,13 @@
         <v>0.9</v>
       </c>
       <c r="AA32" s="2" t="n">
-        <v>70731</v>
+        <v>70620</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>16.412235</v>
+        <v>16.386507</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>12.08132</v>
+        <v>12.062381</v>
       </c>
       <c r="AD32" s="2" t="n">
         <v>11.73</v>
@@ -4803,7 +4803,7 @@
         <v>22.2</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>1.9434006</v>
+        <v>1.9403541</v>
       </c>
       <c r="AI32" s="2" t="n">
         <v>42</v>
@@ -4914,13 +4914,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>542302</v>
+        <v>539400</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>33.765312</v>
+        <v>33.584583</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>21.442049</v>
+        <v>21.32728</v>
       </c>
       <c r="AD33" s="4" t="n">
         <v>16.95</v>
@@ -4935,7 +4935,7 @@
         <v>-34.5</v>
       </c>
       <c r="AH33" s="4" t="n">
-        <v>4.9619246</v>
+        <v>4.9353657</v>
       </c>
       <c r="AI33" s="4" t="n">
         <v>97</v>
@@ -5048,13 +5048,13 @@
         <v>0.86</v>
       </c>
       <c r="AA34" s="2" t="n">
-        <v>251289</v>
+        <v>249315</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>65.54889</v>
+        <v>65.03375</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>52.329422</v>
+        <v>51.91818</v>
       </c>
       <c r="AD34" s="2" t="inlineStr"/>
       <c r="AE34" s="2" t="n">
@@ -5067,7 +5067,7 @@
         <v>-4.6</v>
       </c>
       <c r="AH34" s="2" t="n">
-        <v>12.82813</v>
+        <v>12.727317</v>
       </c>
       <c r="AI34" s="2" t="n">
         <v>96</v>
@@ -5178,13 +5178,13 @@
         <v>0.6</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>367175</v>
+        <v>363866</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>72.466736</v>
+        <v>71.81373000000001</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>48.085255</v>
+        <v>47.65195</v>
       </c>
       <c r="AD35" s="4" t="n">
         <v>37.13</v>
@@ -5199,7 +5199,7 @@
         <v>35.1</v>
       </c>
       <c r="AH35" s="4" t="n">
-        <v>28.670078</v>
+        <v>28.411728</v>
       </c>
       <c r="AI35" s="4" t="n">
         <v>26</v>
@@ -5312,13 +5312,13 @@
         <v>0.49</v>
       </c>
       <c r="AA36" s="2" t="n">
-        <v>274894</v>
+        <v>276257</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>92.37563</v>
+        <v>92.83365999999999</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>59.4446</v>
+        <v>59.739346</v>
       </c>
       <c r="AD36" s="2" t="n">
         <v>12.94</v>
@@ -5333,7 +5333,7 @@
         <v>19.6</v>
       </c>
       <c r="AH36" s="2" t="n">
-        <v>11.211924</v>
+        <v>11.267516</v>
       </c>
       <c r="AI36" s="2" t="n">
         <v>0</v>
@@ -5446,13 +5446,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>143026</v>
+        <v>142432</v>
       </c>
       <c r="AB37" s="4" t="n">
-        <v>5.5224257</v>
+        <v>5.4994903</v>
       </c>
       <c r="AC37" s="4" t="n">
-        <v>6.6577044</v>
+        <v>6.630054</v>
       </c>
       <c r="AD37" s="4" t="n">
         <v>20.47</v>
@@ -5467,7 +5467,7 @@
         <v>10.8</v>
       </c>
       <c r="AH37" s="4" t="n">
-        <v>1.0764304</v>
+        <v>1.0719599</v>
       </c>
       <c r="AI37" s="4" t="n">
         <v>340</v>
@@ -5580,13 +5580,13 @@
         <v>0.87</v>
       </c>
       <c r="AA38" s="2" t="n">
-        <v>379867</v>
+        <v>377588</v>
       </c>
       <c r="AB38" s="2" t="n">
-        <v>21.691584</v>
+        <v>21.561462</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>14.632711</v>
+        <v>14.544933</v>
       </c>
       <c r="AD38" s="2" t="inlineStr"/>
       <c r="AE38" s="2" t="n">
@@ -5599,7 +5599,7 @@
         <v>-1.6</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>1.9763296</v>
+        <v>1.9644741</v>
       </c>
       <c r="AI38" s="2" t="n">
         <v>292</v>
@@ -5706,13 +5706,13 @@
         <v>0.75</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>39051</v>
+        <v>38925</v>
       </c>
       <c r="AB39" s="4" t="n">
-        <v>72.89869</v>
+        <v>72.66298999999999</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>42.94922</v>
+        <v>42.81035</v>
       </c>
       <c r="AD39" s="4" t="n">
         <v>13.8</v>
@@ -5727,7 +5727,7 @@
         <v>18.9</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>10.337079</v>
+        <v>10.303656</v>
       </c>
       <c r="AI39" s="4" t="n">
         <v>24</v>
@@ -5840,13 +5840,13 @@
         <v>0.8</v>
       </c>
       <c r="AA40" s="2" t="n">
-        <v>132894</v>
+        <v>132607</v>
       </c>
       <c r="AB40" s="2" t="n">
-        <v>35.456097</v>
+        <v>35.37937</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>27.500029</v>
+        <v>27.44052</v>
       </c>
       <c r="AD40" s="2" t="n">
         <v>11.34</v>
@@ -5861,10 +5861,10 @@
         <v>-4.6</v>
       </c>
       <c r="AH40" s="2" t="n">
-        <v>3.5102673</v>
+        <v>3.5026712</v>
       </c>
       <c r="AI40" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AJ40" s="2" t="n">
         <v>0.806</v>
@@ -5974,13 +5974,13 @@
         <v>0.74</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>189263</v>
+        <v>188797</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>35.391125</v>
+        <v>35.303925</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>29.976454</v>
+        <v>29.902594</v>
       </c>
       <c r="AD41" s="4" t="inlineStr"/>
       <c r="AE41" s="4" t="n">
@@ -5993,7 +5993,7 @@
         <v>21.3</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>8.568083</v>
+        <v>8.546970999999999</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>101</v>
@@ -6598,13 +6598,13 @@
         <v>0.59</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>139854</v>
+        <v>137942</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.590015</v>
+        <v>51.87985</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.749046</v>
+        <v>37.232964</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -6619,7 +6619,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.6461735</v>
+        <v>11.486955</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -6732,13 +6732,13 @@
         <v>1.14</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>183213</v>
+        <v>183492</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>73.70247999999999</v>
+        <v>73.81461</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>59.035583</v>
+        <v>59.1254</v>
       </c>
       <c r="AD3" s="4" t="inlineStr"/>
       <c r="AE3" s="4" t="n">
@@ -6751,7 +6751,7 @@
         <v>-1</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>11.879639</v>
+        <v>11.897712</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>44</v>
@@ -6862,13 +6862,13 @@
         <v>0.73</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>411487</v>
+        <v>406142</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>30.645163</v>
+        <v>30.247084</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>23.027498</v>
+        <v>22.728373</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>15.59</v>
@@ -6883,7 +6883,7 @@
         <v>3.6</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>4.280397</v>
+        <v>4.2247953</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>42</v>
@@ -6996,13 +6996,13 @@
         <v>1.55</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>315135</v>
+        <v>313670</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>14.140839</v>
+        <v>14.081297</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>17.93597</v>
+        <v>17.852625</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>27.26</v>
@@ -7017,7 +7017,7 @@
         <v>991.8</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>3.149806</v>
+        <v>3.1351693</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>55</v>
@@ -7130,13 +7130,13 @@
         <v>4.31</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>12643</v>
+        <v>12734</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>30.567175</v>
+        <v>30.785805</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>18.259304</v>
+        <v>18.389902</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>10.66</v>
@@ -7151,7 +7151,7 @@
         <v>5.9</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>3.2903805</v>
+        <v>3.3139148</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>79</v>
@@ -7264,13 +7264,13 @@
         <v>0.82</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>107778</v>
+        <v>107740</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>61.20309</v>
+        <v>61.181015</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>44.07573</v>
+        <v>44.059834</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>41.39</v>
@@ -7285,7 +7285,7 @@
         <v>14.5</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>25.410913</v>
+        <v>25.401749</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>48</v>
@@ -7645,13 +7645,13 @@
         <v>0.59</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>139854</v>
+        <v>137942</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.590015</v>
+        <v>51.87985</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.749046</v>
+        <v>37.232964</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -7666,7 +7666,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.6461735</v>
+        <v>11.486955</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -7779,13 +7779,13 @@
         <v>1.14</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>183213</v>
+        <v>183492</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>73.70247999999999</v>
+        <v>73.81461</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>59.035583</v>
+        <v>59.1254</v>
       </c>
       <c r="AD3" s="4" t="inlineStr"/>
       <c r="AE3" s="4" t="n">
@@ -7798,7 +7798,7 @@
         <v>-1</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>11.879639</v>
+        <v>11.897712</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>44</v>
@@ -7909,13 +7909,13 @@
         <v>0.73</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>411487</v>
+        <v>406142</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>30.645163</v>
+        <v>30.247084</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>23.027498</v>
+        <v>22.728373</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>15.59</v>
@@ -7930,7 +7930,7 @@
         <v>3.6</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>4.280397</v>
+        <v>4.2247953</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>42</v>
@@ -8043,13 +8043,13 @@
         <v>1.55</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>315135</v>
+        <v>313670</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>14.140839</v>
+        <v>14.081297</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>17.93597</v>
+        <v>17.852625</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>27.26</v>
@@ -8064,7 +8064,7 @@
         <v>991.8</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>3.149806</v>
+        <v>3.1351693</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>55</v>
@@ -8177,13 +8177,13 @@
         <v>4.31</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>12643</v>
+        <v>12734</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>30.567175</v>
+        <v>30.785805</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>18.259304</v>
+        <v>18.389902</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>10.66</v>
@@ -8198,7 +8198,7 @@
         <v>5.9</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>3.2903805</v>
+        <v>3.3139148</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>79</v>
@@ -8311,13 +8311,13 @@
         <v>0.82</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>107778</v>
+        <v>107740</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>61.20309</v>
+        <v>61.181015</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>44.07573</v>
+        <v>44.059834</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>41.39</v>
@@ -8332,7 +8332,7 @@
         <v>14.5</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>25.410913</v>
+        <v>25.401749</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>48</v>
@@ -8377,7 +8377,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 19-May-2026 07:00 IST</t>
+          <t>Run Date: 19-May-2026 12:02 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>

</xml_diff>

<commit_message>
📈 Daily Screener Report — 19-May-2026 18:11 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -1354,7 +1354,7 @@
         <v>30.785805</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>18.389902</v>
+        <v>18.240303</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>10.66</v>
@@ -5712,7 +5712,7 @@
         <v>72.66298999999999</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>42.81035</v>
+        <v>42.825382</v>
       </c>
       <c r="AD39" s="4" t="n">
         <v>13.8</v>
@@ -7136,7 +7136,7 @@
         <v>30.785805</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>18.389902</v>
+        <v>18.240303</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>10.66</v>
@@ -8183,7 +8183,7 @@
         <v>30.785805</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>18.389902</v>
+        <v>18.240303</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>10.66</v>
@@ -8377,7 +8377,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 19-May-2026 12:02 IST</t>
+          <t>Run Date: 19-May-2026 12:41 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>

</xml_diff>

<commit_message>
📈 Daily Screener Report — 19-May-2026 23:47 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -2018,7 +2018,7 @@
         <v>80.46856</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>41.54123</v>
+        <v>41.47935</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -8377,7 +8377,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 19-May-2026 12:41 IST</t>
+          <t>Run Date: 19-May-2026 18:17 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>

</xml_diff>

<commit_message>
📈 Daily Screener Report — 20-May-2026 13:08 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -816,13 +816,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>138582</v>
+        <v>138634</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.052704</v>
+        <v>52.072495</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.40567</v>
+        <v>37.41989</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -837,7 +837,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.540236</v>
+        <v>11.544624</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -950,13 +950,13 @@
         <v>0.66</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>407110</v>
+        <v>405981</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>30.376484</v>
+        <v>30.292248</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>22.782524</v>
+        <v>22.719347</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>15.59</v>
@@ -971,7 +971,7 @@
         <v>3.6</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.234861</v>
+        <v>4.2231174</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>43</v>
@@ -1084,13 +1084,13 @@
         <v>1.06</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>183041</v>
+        <v>182775</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>73.89348</v>
+        <v>73.78631</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>58.979984</v>
+        <v>58.894444</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="n">
@@ -1103,7 +1103,7 @@
         <v>-1</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>11.86845</v>
+        <v>11.851236</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>43</v>
@@ -1214,13 +1214,13 @@
         <v>0.77</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>107856</v>
+        <v>108076</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>61.428043</v>
+        <v>61.553505</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>44.107525</v>
+        <v>44.19761</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>41.39</v>
@@ -1235,7 +1235,7 @@
         <v>14.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>25.429243</v>
+        <v>25.481182</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>48</v>
@@ -1348,13 +1348,13 @@
         <v>0.75</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>271912</v>
+        <v>271873</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>77.563255</v>
+        <v>77.55225</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>59.524837</v>
+        <v>59.5164</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>76.34</v>
@@ -1369,7 +1369,7 @@
         <v>27.4</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>52.727818</v>
+        <v>52.72034</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>84</v>
@@ -1482,11 +1482,11 @@
         <v>0.09</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>3297</v>
+        <v>3284</v>
       </c>
       <c r="AB7" s="4" t="inlineStr"/>
       <c r="AC7" s="4" t="n">
-        <v>27.240143</v>
+        <v>27.132616</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>-2.82</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="AG7" s="4" t="inlineStr"/>
       <c r="AH7" s="4" t="n">
-        <v>5.547567</v>
+        <v>5.5256686</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>0</v>
@@ -1612,13 +1612,13 @@
         <v>0.55</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>377031</v>
+        <v>376276</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>9.910715</v>
+        <v>9.890872999999999</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>7.0774803</v>
+        <v>7.063311</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
@@ -1631,7 +1631,7 @@
         <v>16.2</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>1.0243038</v>
+        <v>1.0222532</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>624</v>
@@ -1742,13 +1742,13 @@
         <v>0.82</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>9758</v>
+        <v>9968</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>86.86682999999999</v>
+        <v>88.73365</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>44.671246</v>
+        <v>45.63126</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -1761,7 +1761,7 @@
         <v>35.8</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>14.970593</v>
+        <v>15.292321</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>0</v>
@@ -1872,13 +1872,13 @@
         <v>1.32</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>371005</v>
+        <v>370799</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>36.779015</v>
+        <v>36.75863</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>47.741024</v>
+        <v>47.71456</v>
       </c>
       <c r="AD10" s="2" t="n">
         <v>13.66</v>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="AG10" s="2" t="inlineStr"/>
       <c r="AH10" s="2" t="n">
-        <v>4.3161635</v>
+        <v>4.3137712</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>5</v>
@@ -2004,13 +2004,13 @@
         <v>0.41</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>450067</v>
+        <v>450307</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>41.18112</v>
+        <v>41.203075</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>33.151623</v>
+        <v>33.169296</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -2023,7 +2023,7 @@
         <v>15.7</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>5.7812624</v>
+        <v>5.7843447</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>88</v>
@@ -2134,13 +2134,13 @@
         <v>0.61</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>310497</v>
+        <v>311278</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>13.941917</v>
+        <v>13.976987</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>17.644154</v>
+        <v>17.688536</v>
       </c>
       <c r="AD12" s="2" t="n">
         <v>27.26</v>
@@ -2155,7 +2155,7 @@
         <v>991.8</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>3.1034567</v>
+        <v>3.111263</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>55</v>
@@ -2268,13 +2268,13 @@
         <v>1.03</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>115919</v>
+        <v>116336</v>
       </c>
       <c r="AB13" s="4" t="n">
-        <v>64.38782999999999</v>
+        <v>64.61944</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>48.4503</v>
+        <v>48.62458</v>
       </c>
       <c r="AD13" s="4" t="inlineStr"/>
       <c r="AE13" s="4" t="n">
@@ -2287,7 +2287,7 @@
         <v>35</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>12.747192</v>
+        <v>12.793045</v>
       </c>
       <c r="AI13" s="4" t="n">
         <v>25</v>
@@ -2398,13 +2398,13 @@
         <v>1.09</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>149166</v>
+        <v>149501</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>65.88042</v>
+        <v>66.0284</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>68.05428999999999</v>
+        <v>68.20715</v>
       </c>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="n">
@@ -2417,7 +2417,7 @@
         <v>26.1</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>17.667267</v>
+        <v>17.706951</v>
       </c>
       <c r="AI14" s="2" t="n">
         <v>78</v>
@@ -2528,13 +2528,13 @@
         <v>0.4</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>23966</v>
+        <v>23839</v>
       </c>
       <c r="AB15" s="4" t="n">
-        <v>15.559381</v>
+        <v>15.476764</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>12.633947</v>
+        <v>12.566864</v>
       </c>
       <c r="AD15" s="4" t="n">
         <v>12.55</v>
@@ -2549,7 +2549,7 @@
         <v>17.8</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>1.8832353</v>
+        <v>1.8732358</v>
       </c>
       <c r="AI15" s="4" t="n">
         <v>331</v>
@@ -2662,13 +2662,13 @@
         <v>1.24</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>87688</v>
+        <v>87457</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>25.374624</v>
+        <v>25.308025</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>19.942963</v>
+        <v>19.89062</v>
       </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="n">
@@ -2681,7 +2681,7 @@
         <v>7.6</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>2.5257087</v>
+        <v>2.5190794</v>
       </c>
       <c r="AI16" s="2" t="n">
         <v>26</v>
@@ -2792,13 +2792,13 @@
         <v>0.78</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>12929</v>
+        <v>12920</v>
       </c>
       <c r="AB17" s="4" t="n">
-        <v>31.238125</v>
+        <v>30.369686</v>
       </c>
       <c r="AC17" s="4" t="n">
-        <v>18.520027</v>
+        <v>18.506886</v>
       </c>
       <c r="AD17" s="4" t="n">
         <v>10.66</v>
@@ -2813,7 +2813,7 @@
         <v>5.9</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>3.1932802</v>
+        <v>3.3623478</v>
       </c>
       <c r="AI17" s="4" t="n">
         <v>77</v>
@@ -2926,13 +2926,13 @@
         <v>0.68</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>30298</v>
+        <v>30157</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>27.568375</v>
+        <v>27.44017</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>10.98354</v>
+        <v>10.932461</v>
       </c>
       <c r="AD18" s="2" t="n">
         <v>6.97</v>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="n">
-        <v>1.6822258</v>
+        <v>1.6744027</v>
       </c>
       <c r="AI18" s="2" t="n">
         <v>63</v>
@@ -3058,13 +3058,13 @@
         <v>0.7</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>77587</v>
+        <v>77429</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>552.95917</v>
+        <v>551.83673</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>174.6915</v>
+        <v>174.33688</v>
       </c>
       <c r="AD19" s="4" t="inlineStr"/>
       <c r="AE19" s="4" t="n">
@@ -3077,7 +3077,7 @@
         <v>144.4</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>56.01613</v>
+        <v>55.90242</v>
       </c>
       <c r="AI19" s="4" t="n">
         <v>0</v>
@@ -3188,13 +3188,13 @@
         <v>0.42</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>20021</v>
+        <v>19975</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>22.982956</v>
+        <v>22.929688</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>17.051458</v>
+        <v>17.011938</v>
       </c>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
@@ -3205,7 +3205,7 @@
         <v>367.9</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>1.1959891</v>
+        <v>1.1932173</v>
       </c>
       <c r="AI20" s="2" t="n">
         <v>33</v>
@@ -3316,13 +3316,13 @@
         <v>0.37</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>59221</v>
+        <v>59198</v>
       </c>
       <c r="AB21" s="4" t="n">
-        <v>52.632126</v>
+        <v>52.6114</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>39.99534</v>
+        <v>39.979588</v>
       </c>
       <c r="AD21" s="4" t="n">
         <v>17.23</v>
@@ -3337,7 +3337,7 @@
         <v>27.7</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>8.565935</v>
+        <v>8.562563000000001</v>
       </c>
       <c r="AI21" s="4" t="n">
         <v>75</v>
@@ -3450,13 +3450,13 @@
         <v>0.46</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>18912</v>
+        <v>18869</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>57.99173</v>
+        <v>57.85883</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>34.514725</v>
+        <v>34.435627</v>
       </c>
       <c r="AD22" s="2" t="n">
         <v>14.14</v>
@@ -3471,7 +3471,7 @@
         <v>43.7</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>6.5090127</v>
+        <v>6.494096</v>
       </c>
       <c r="AI22" s="2" t="n">
         <v>15</v>
@@ -3584,13 +3584,13 @@
         <v>0.27</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>30696</v>
+        <v>30605</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>25.104082</v>
+        <v>25.028986</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>8.811726</v>
+        <v>8.785365000000001</v>
       </c>
       <c r="AD23" s="4" t="n">
         <v>4.88</v>
@@ -3603,7 +3603,7 @@
         <v>68</v>
       </c>
       <c r="AH23" s="4" t="n">
-        <v>1.198636</v>
+        <v>1.1950505</v>
       </c>
       <c r="AI23" s="4" t="n">
         <v>78</v>
@@ -3714,13 +3714,13 @@
         <v>0.57</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>21590</v>
+        <v>21499</v>
       </c>
       <c r="AB24" s="2" t="n">
-        <v>391.91663</v>
+        <v>390.25</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>27.132692</v>
+        <v>27.01731</v>
       </c>
       <c r="AD24" s="2" t="n">
         <v>7.27</v>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="AG24" s="2" t="inlineStr"/>
       <c r="AH24" s="2" t="n">
-        <v>4.3546295</v>
+        <v>4.336111</v>
       </c>
       <c r="AI24" s="2" t="n">
         <v>7</v>
@@ -3846,13 +3846,13 @@
         <v>0.74</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>110602</v>
+        <v>110502</v>
       </c>
       <c r="AB25" s="4" t="n">
-        <v>26.388557</v>
+        <v>26.36472</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>20.700478</v>
+        <v>20.681778</v>
       </c>
       <c r="AD25" s="4" t="n">
         <v>11.83</v>
@@ -3867,7 +3867,7 @@
         <v>-86.2</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>2.9371836</v>
+        <v>2.9345303</v>
       </c>
       <c r="AI25" s="4" t="n">
         <v>60</v>
@@ -3980,13 +3980,13 @@
         <v>0.86</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>70731</v>
+        <v>70830</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>16.421625</v>
+        <v>16.44451</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>12.08132</v>
+        <v>12.098156</v>
       </c>
       <c r="AD26" s="2" t="n">
         <v>11.73</v>
@@ -3999,7 +3999,7 @@
         <v>22.2</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>1.9434006</v>
+        <v>1.9461088</v>
       </c>
       <c r="AI26" s="2" t="n">
         <v>42</v>
@@ -4110,13 +4110,13 @@
         <v>0.61</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>113544</v>
+        <v>113682</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>29.3261</v>
+        <v>29.36157</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>22.188253</v>
+        <v>22.215092</v>
       </c>
       <c r="AD27" s="4" t="n">
         <v>11.74</v>
@@ -4131,7 +4131,7 @@
         <v>-54.6</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>3.4490626</v>
+        <v>3.4532342</v>
       </c>
       <c r="AI27" s="4" t="n">
         <v>92</v>
@@ -4244,13 +4244,13 @@
         <v>0.65</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>281976</v>
+        <v>282838</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>9.069375000000001</v>
+        <v>9.097125999999999</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>8.000878999999999</v>
+        <v>8.025361</v>
       </c>
       <c r="AD28" s="2" t="n">
         <v>28.12</v>
@@ -4265,7 +4265,7 @@
         <v>12.9</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>2.367291</v>
+        <v>2.3745344</v>
       </c>
       <c r="AI28" s="2" t="n">
         <v>481</v>
@@ -4378,13 +4378,13 @@
         <v>0.57</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>148158</v>
+        <v>147893</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>60.60366</v>
+        <v>60.49542</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>48.02086</v>
+        <v>47.93509</v>
       </c>
       <c r="AD29" s="4" t="n">
         <v>23.52</v>
@@ -4399,7 +4399,7 @@
         <v>37</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>15.511251</v>
+        <v>15.483547</v>
       </c>
       <c r="AI29" s="4" t="n">
         <v>69</v>
@@ -4512,13 +4512,13 @@
         <v>1.16</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>255186</v>
+        <v>255211</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>27.838097</v>
+        <v>27.840816</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>10.883512</v>
+        <v>10.884575</v>
       </c>
       <c r="AD30" s="2" t="n">
         <v>11.16</v>
@@ -4533,7 +4533,7 @@
         <v>125.4</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>2.6844308</v>
+        <v>2.6846933</v>
       </c>
       <c r="AI30" s="2" t="n">
         <v>191</v>
@@ -4646,13 +4646,13 @@
         <v>1.3</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>276693</v>
+        <v>277297</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>14.778937</v>
+        <v>14.811228</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>14.924811</v>
+        <v>14.957419</v>
       </c>
       <c r="AD31" s="4" t="n">
         <v>16.49</v>
@@ -4667,7 +4667,7 @@
         <v>9.6</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>2.7926145</v>
+        <v>2.7987158</v>
       </c>
       <c r="AI31" s="4" t="n">
         <v>410</v>
@@ -4780,13 +4780,13 @@
         <v>0.91</v>
       </c>
       <c r="AA32" s="2" t="n">
-        <v>538712</v>
+        <v>538326</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>33.51305</v>
+        <v>33.48909</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>21.300083</v>
+        <v>21.284853</v>
       </c>
       <c r="AD32" s="2" t="n">
         <v>16.95</v>
@@ -4801,7 +4801,7 @@
         <v>-34.5</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>4.9290724</v>
+        <v>4.925548</v>
       </c>
       <c r="AI32" s="2" t="n">
         <v>97</v>
@@ -4914,13 +4914,13 @@
         <v>1.07</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>269578</v>
+        <v>269083</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>90.35191</v>
+        <v>90.18579</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>58.295223</v>
+        <v>58.188038</v>
       </c>
       <c r="AD33" s="4" t="n">
         <v>12.94</v>
@@ -4935,7 +4935,7 @@
         <v>19.6</v>
       </c>
       <c r="AH33" s="4" t="n">
-        <v>10.995138</v>
+        <v>10.974922</v>
       </c>
       <c r="AI33" s="4" t="n">
         <v>0</v>
@@ -5048,13 +5048,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA34" s="2" t="n">
-        <v>249104</v>
+        <v>250254</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>64.8814</v>
+        <v>65.18102</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>51.87426</v>
+        <v>52.11382</v>
       </c>
       <c r="AD34" s="2" t="inlineStr"/>
       <c r="AE34" s="2" t="n">
@@ -5067,7 +5067,7 @@
         <v>-4.6</v>
       </c>
       <c r="AH34" s="2" t="n">
-        <v>12.716551</v>
+        <v>12.775277</v>
       </c>
       <c r="AI34" s="2" t="n">
         <v>96</v>
@@ -5178,13 +5178,13 @@
         <v>1.12</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>131878</v>
+        <v>132139</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>12.460266</v>
+        <v>12.484921</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>9.512487</v>
+        <v>9.53131</v>
       </c>
       <c r="AD35" s="4" t="n">
         <v>30.41</v>
@@ -5199,7 +5199,7 @@
         <v>126.7</v>
       </c>
       <c r="AH35" s="4" t="n">
-        <v>3.7022343</v>
+        <v>3.70956</v>
       </c>
       <c r="AI35" s="4" t="n">
         <v>91</v>
@@ -5312,13 +5312,13 @@
         <v>0.5</v>
       </c>
       <c r="AA36" s="2" t="n">
-        <v>362668</v>
+        <v>361835</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>71.70291</v>
+        <v>71.538055</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>47.495125</v>
+        <v>47.38593</v>
       </c>
       <c r="AD36" s="2" t="n">
         <v>37.13</v>
@@ -5333,7 +5333,7 @@
         <v>35.1</v>
       </c>
       <c r="AH36" s="2" t="n">
-        <v>28.318222</v>
+        <v>28.253117</v>
       </c>
       <c r="AI36" s="2" t="n">
         <v>27</v>
@@ -5442,13 +5442,13 @@
         <v>1.38</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>32654</v>
+        <v>32546</v>
       </c>
       <c r="AB37" s="4" t="n">
-        <v>37.607494</v>
+        <v>37.483234</v>
       </c>
       <c r="AC37" s="4" t="n">
-        <v>26.450455</v>
+        <v>26.36306</v>
       </c>
       <c r="AD37" s="4" t="inlineStr"/>
       <c r="AE37" s="4" t="n">
@@ -5461,7 +5461,7 @@
         <v>3</v>
       </c>
       <c r="AH37" s="4" t="n">
-        <v>6.092783</v>
+        <v>6.072652</v>
       </c>
       <c r="AI37" s="4" t="n">
         <v>54</v>
@@ -5572,13 +5572,13 @@
         <v>0.61</v>
       </c>
       <c r="AA38" s="2" t="n">
-        <v>141277</v>
+        <v>140419</v>
       </c>
       <c r="AB38" s="2" t="n">
-        <v>5.4528084</v>
+        <v>5.4196916</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>6.576288</v>
+        <v>6.5363483</v>
       </c>
       <c r="AD38" s="2" t="n">
         <v>20.47</v>
@@ -5593,7 +5593,7 @@
         <v>10.8</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>1.063267</v>
+        <v>1.0568094</v>
       </c>
       <c r="AI38" s="2" t="n">
         <v>338</v>
@@ -5706,13 +5706,13 @@
         <v>1.01</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>131664</v>
+        <v>131696</v>
       </c>
       <c r="AB39" s="4" t="n">
-        <v>35.21795</v>
+        <v>35.226498</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>27.24546</v>
+        <v>27.252073</v>
       </c>
       <c r="AD39" s="4" t="n">
         <v>11.34</v>
@@ -5727,7 +5727,7 @@
         <v>-4.6</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>3.4777727</v>
+        <v>3.4786167</v>
       </c>
       <c r="AI39" s="4" t="n">
         <v>60</v>
@@ -5840,13 +5840,13 @@
         <v>0.78</v>
       </c>
       <c r="AA40" s="2" t="n">
-        <v>378800</v>
+        <v>379382</v>
       </c>
       <c r="AB40" s="2" t="n">
-        <v>21.618706</v>
+        <v>21.651909</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>14.591623</v>
+        <v>14.614035</v>
       </c>
       <c r="AD40" s="2" t="inlineStr"/>
       <c r="AE40" s="2" t="n">
@@ -5859,7 +5859,7 @@
         <v>-1.6</v>
       </c>
       <c r="AH40" s="2" t="n">
-        <v>1.9707801</v>
+        <v>1.9738071</v>
       </c>
       <c r="AI40" s="2" t="n">
         <v>291</v>
@@ -5970,13 +5970,13 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>188358</v>
+        <v>188605</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>35.254402</v>
+        <v>35.30061</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>29.833076</v>
+        <v>29.872179</v>
       </c>
       <c r="AD41" s="4" t="inlineStr"/>
       <c r="AE41" s="4" t="n">
@@ -5989,7 +5989,7 @@
         <v>21.3</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>8.527101999999999</v>
+        <v>8.538278999999999</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>102</v>
@@ -6594,13 +6594,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>138582</v>
+        <v>138634</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.052704</v>
+        <v>52.072495</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.40567</v>
+        <v>37.41989</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -6615,7 +6615,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.540236</v>
+        <v>11.544624</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -6728,13 +6728,13 @@
         <v>0.66</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>407110</v>
+        <v>405981</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>30.376484</v>
+        <v>30.292248</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>22.782524</v>
+        <v>22.719347</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>15.59</v>
@@ -6749,7 +6749,7 @@
         <v>3.6</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.234861</v>
+        <v>4.2231174</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>43</v>
@@ -6862,13 +6862,13 @@
         <v>1.06</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>183041</v>
+        <v>182775</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>73.89348</v>
+        <v>73.78631</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>58.979984</v>
+        <v>58.894444</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="n">
@@ -6881,7 +6881,7 @@
         <v>-1</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>11.86845</v>
+        <v>11.851236</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>43</v>
@@ -6992,13 +6992,13 @@
         <v>0.77</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>107856</v>
+        <v>108076</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>61.428043</v>
+        <v>61.553505</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>44.107525</v>
+        <v>44.19761</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>41.39</v>
@@ -7013,7 +7013,7 @@
         <v>14.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>25.429243</v>
+        <v>25.481182</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>48</v>
@@ -7373,13 +7373,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>138582</v>
+        <v>138634</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.052704</v>
+        <v>52.072495</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.40567</v>
+        <v>37.41989</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -7394,7 +7394,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.540236</v>
+        <v>11.544624</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -7507,13 +7507,13 @@
         <v>0.66</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>407110</v>
+        <v>405981</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>30.376484</v>
+        <v>30.292248</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>22.782524</v>
+        <v>22.719347</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>15.59</v>
@@ -7528,7 +7528,7 @@
         <v>3.6</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.234861</v>
+        <v>4.2231174</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>43</v>
@@ -7641,13 +7641,13 @@
         <v>1.06</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>183041</v>
+        <v>182775</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>73.89348</v>
+        <v>73.78631</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>58.979984</v>
+        <v>58.894444</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="n">
@@ -7660,7 +7660,7 @@
         <v>-1</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>11.86845</v>
+        <v>11.851236</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>43</v>
@@ -7771,13 +7771,13 @@
         <v>0.77</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>107856</v>
+        <v>108076</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>61.428043</v>
+        <v>61.553505</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>44.107525</v>
+        <v>44.19761</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>41.39</v>
@@ -7792,7 +7792,7 @@
         <v>14.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>25.429243</v>
+        <v>25.481182</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>48</v>
@@ -7837,7 +7837,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 20-May-2026 07:00 IST</t>
+          <t>Run Date: 20-May-2026 07:38 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>

</xml_diff>

<commit_message>
📈 Daily Screener Report — 20-May-2026 15:25 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -517,7 +517,7 @@
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="17" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
     <col width="8" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
@@ -816,13 +816,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>138634</v>
+        <v>138476</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.072495</v>
+        <v>52.01312</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.41989</v>
+        <v>37.377224</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -837,7 +837,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.544624</v>
+        <v>11.531461</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -950,13 +950,13 @@
         <v>0.66</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>405981</v>
+        <v>408492</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>30.292248</v>
+        <v>30.47963</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>22.719347</v>
+        <v>22.859884</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>15.59</v>
@@ -971,7 +971,7 @@
         <v>3.6</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.2231174</v>
+        <v>4.249241</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>43</v>
@@ -1214,13 +1214,13 @@
         <v>0.77</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>108076</v>
+        <v>108711</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>61.553505</v>
+        <v>61.91513</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>44.19761</v>
+        <v>44.45727</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>41.39</v>
@@ -1235,7 +1235,7 @@
         <v>14.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>25.481182</v>
+        <v>25.630882</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>48</v>
@@ -1348,13 +1348,13 @@
         <v>0.75</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>271873</v>
+        <v>274052</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>77.55225</v>
+        <v>78.17381</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>59.5164</v>
+        <v>59.993404</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>76.34</v>
@@ -1369,7 +1369,7 @@
         <v>27.4</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>52.72034</v>
+        <v>53.142876</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>84</v>
@@ -1482,11 +1482,11 @@
         <v>0.09</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>3284</v>
+        <v>3263</v>
       </c>
       <c r="AB7" s="4" t="inlineStr"/>
       <c r="AC7" s="4" t="n">
-        <v>27.132616</v>
+        <v>26.953405</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>-2.82</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="AG7" s="4" t="inlineStr"/>
       <c r="AH7" s="4" t="n">
-        <v>5.5256686</v>
+        <v>5.4891715</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>0</v>
@@ -1612,13 +1612,13 @@
         <v>0.55</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>376276</v>
+        <v>375710</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>9.890872999999999</v>
+        <v>9.875992</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>7.063311</v>
+        <v>7.052684</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
@@ -1631,7 +1631,7 @@
         <v>16.2</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>1.0222532</v>
+        <v>1.0207151</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>624</v>
@@ -1742,13 +1742,13 @@
         <v>0.82</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>9968</v>
+        <v>9771</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>88.73365</v>
+        <v>86.97978999999999</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>45.63126</v>
+        <v>44.729336</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -1761,7 +1761,7 @@
         <v>35.8</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>15.292321</v>
+        <v>14.990062</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>0</v>
@@ -1872,13 +1872,13 @@
         <v>1.32</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>370799</v>
+        <v>370827</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>36.75863</v>
+        <v>36.761345</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>47.71456</v>
+        <v>47.71809</v>
       </c>
       <c r="AD10" s="2" t="n">
         <v>13.66</v>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="AG10" s="2" t="inlineStr"/>
       <c r="AH10" s="2" t="n">
-        <v>4.3137712</v>
+        <v>4.31409</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>5</v>
@@ -2004,13 +2004,13 @@
         <v>0.41</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>450307</v>
+        <v>451195</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>41.203075</v>
+        <v>41.2843</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>33.169296</v>
+        <v>33.234688</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -2023,7 +2023,7 @@
         <v>15.7</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>5.7843447</v>
+        <v>5.7957478</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>88</v>
@@ -2134,13 +2134,13 @@
         <v>0.61</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>311278</v>
+        <v>313206</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>13.976987</v>
+        <v>14.063562</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>17.688536</v>
+        <v>17.798101</v>
       </c>
       <c r="AD12" s="2" t="n">
         <v>27.26</v>
@@ -2155,7 +2155,7 @@
         <v>991.8</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>3.111263</v>
+        <v>3.1305346</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>55</v>
@@ -2268,13 +2268,13 @@
         <v>1.03</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>116336</v>
+        <v>116106</v>
       </c>
       <c r="AB13" s="4" t="n">
-        <v>64.61944</v>
+        <v>64.49165000000001</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>48.62458</v>
+        <v>48.528423</v>
       </c>
       <c r="AD13" s="4" t="inlineStr"/>
       <c r="AE13" s="4" t="n">
@@ -2287,7 +2287,7 @@
         <v>35</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>12.793045</v>
+        <v>12.767747</v>
       </c>
       <c r="AI13" s="4" t="n">
         <v>25</v>
@@ -2398,13 +2398,13 @@
         <v>1.09</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>149501</v>
+        <v>149894</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>66.0284</v>
+        <v>66.20179</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>68.20715</v>
+        <v>68.38627</v>
       </c>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="n">
@@ -2417,7 +2417,7 @@
         <v>26.1</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>17.706951</v>
+        <v>17.75345</v>
       </c>
       <c r="AI14" s="2" t="n">
         <v>78</v>
@@ -2528,13 +2528,13 @@
         <v>0.4</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>23839</v>
+        <v>23940</v>
       </c>
       <c r="AB15" s="4" t="n">
-        <v>15.476764</v>
+        <v>15.54217</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>12.566864</v>
+        <v>12.619972</v>
       </c>
       <c r="AD15" s="4" t="n">
         <v>12.55</v>
@@ -2549,7 +2549,7 @@
         <v>17.8</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>1.8732358</v>
+        <v>1.8811522</v>
       </c>
       <c r="AI15" s="4" t="n">
         <v>331</v>
@@ -2662,13 +2662,13 @@
         <v>1.24</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>87457</v>
+        <v>87250</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>25.308025</v>
+        <v>25.248085</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>19.89062</v>
+        <v>19.843512</v>
       </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="n">
@@ -2681,7 +2681,7 @@
         <v>7.6</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>2.5190794</v>
+        <v>2.5131133</v>
       </c>
       <c r="AI16" s="2" t="n">
         <v>26</v>
@@ -2792,13 +2792,13 @@
         <v>0.78</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>12920</v>
+        <v>12671</v>
       </c>
       <c r="AB17" s="4" t="n">
-        <v>30.369686</v>
+        <v>30.614313</v>
       </c>
       <c r="AC17" s="4" t="n">
-        <v>18.506886</v>
+        <v>18.15019</v>
       </c>
       <c r="AD17" s="4" t="n">
         <v>10.66</v>
@@ -2813,7 +2813,7 @@
         <v>5.9</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>3.3623478</v>
+        <v>3.297543</v>
       </c>
       <c r="AI17" s="4" t="n">
         <v>77</v>
@@ -2926,13 +2926,13 @@
         <v>0.68</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>30157</v>
+        <v>30007</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>27.44017</v>
+        <v>27.303421</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>10.932461</v>
+        <v>10.877978</v>
       </c>
       <c r="AD18" s="2" t="n">
         <v>6.97</v>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="n">
-        <v>1.6744027</v>
+        <v>1.6660582</v>
       </c>
       <c r="AI18" s="2" t="n">
         <v>63</v>
@@ -3058,13 +3058,13 @@
         <v>0.7</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>77429</v>
+        <v>78417</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>551.83673</v>
+        <v>558.87756</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>174.33688</v>
+        <v>176.56123</v>
       </c>
       <c r="AD19" s="4" t="inlineStr"/>
       <c r="AE19" s="4" t="n">
@@ -3077,7 +3077,7 @@
         <v>144.4</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>55.90242</v>
+        <v>56.615673</v>
       </c>
       <c r="AI19" s="4" t="n">
         <v>0</v>
@@ -3188,13 +3188,13 @@
         <v>0.42</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>19975</v>
+        <v>20321</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>22.929688</v>
+        <v>23.327415</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>17.011938</v>
+        <v>17.307018</v>
       </c>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
@@ -3205,7 +3205,7 @@
         <v>367.9</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>1.1932173</v>
+        <v>1.2139143</v>
       </c>
       <c r="AI20" s="2" t="n">
         <v>33</v>
@@ -3316,13 +3316,13 @@
         <v>0.37</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>59198</v>
+        <v>59379</v>
       </c>
       <c r="AB21" s="4" t="n">
-        <v>52.6114</v>
+        <v>52.772022</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>39.979588</v>
+        <v>40.101646</v>
       </c>
       <c r="AD21" s="4" t="n">
         <v>17.23</v>
@@ -3337,7 +3337,7 @@
         <v>27.7</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>8.562563000000001</v>
+        <v>8.588704</v>
       </c>
       <c r="AI21" s="4" t="n">
         <v>75</v>
@@ -3450,13 +3450,13 @@
         <v>0.46</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>18869</v>
+        <v>19406</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>57.85883</v>
+        <v>59.506794</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>34.435627</v>
+        <v>35.41644</v>
       </c>
       <c r="AD22" s="2" t="n">
         <v>14.14</v>
@@ -3471,7 +3471,7 @@
         <v>43.7</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>6.494096</v>
+        <v>6.679064</v>
       </c>
       <c r="AI22" s="2" t="n">
         <v>15</v>
@@ -3584,13 +3584,13 @@
         <v>0.27</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>30605</v>
+        <v>31044</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>25.028986</v>
+        <v>25.388668</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>8.785365000000001</v>
+        <v>8.911617</v>
       </c>
       <c r="AD23" s="4" t="n">
         <v>4.88</v>
@@ -3603,7 +3603,7 @@
         <v>68</v>
       </c>
       <c r="AH23" s="4" t="n">
-        <v>1.1950505</v>
+        <v>1.2122241</v>
       </c>
       <c r="AI23" s="4" t="n">
         <v>78</v>
@@ -3714,13 +3714,13 @@
         <v>0.57</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>21499</v>
+        <v>21385</v>
       </c>
       <c r="AB24" s="2" t="n">
-        <v>390.25</v>
+        <v>388.19443</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>27.01731</v>
+        <v>26.875002</v>
       </c>
       <c r="AD24" s="2" t="n">
         <v>7.27</v>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="AG24" s="2" t="inlineStr"/>
       <c r="AH24" s="2" t="n">
-        <v>4.336111</v>
+        <v>4.3132715</v>
       </c>
       <c r="AI24" s="2" t="n">
         <v>7</v>
@@ -3846,13 +3846,13 @@
         <v>0.74</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>110502</v>
+        <v>109944</v>
       </c>
       <c r="AB25" s="4" t="n">
-        <v>26.36472</v>
+        <v>26.231625</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>20.681778</v>
+        <v>20.577372</v>
       </c>
       <c r="AD25" s="4" t="n">
         <v>11.83</v>
@@ -3867,7 +3867,7 @@
         <v>-86.2</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>2.9345303</v>
+        <v>2.9197161</v>
       </c>
       <c r="AI25" s="4" t="n">
         <v>60</v>
@@ -3980,13 +3980,13 @@
         <v>0.86</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>70830</v>
+        <v>71470</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>16.44451</v>
+        <v>16.593248</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>12.098156</v>
+        <v>12.207583</v>
       </c>
       <c r="AD26" s="2" t="n">
         <v>11.73</v>
@@ -3999,7 +3999,7 @@
         <v>22.2</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>1.9461088</v>
+        <v>1.9637114</v>
       </c>
       <c r="AI26" s="2" t="n">
         <v>42</v>
@@ -4110,13 +4110,13 @@
         <v>0.61</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>113682</v>
+        <v>112987</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>29.36157</v>
+        <v>29.18214</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>22.215092</v>
+        <v>22.079332</v>
       </c>
       <c r="AD27" s="4" t="n">
         <v>11.74</v>
@@ -4131,7 +4131,7 @@
         <v>-54.6</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>3.4532342</v>
+        <v>3.4321313</v>
       </c>
       <c r="AI27" s="4" t="n">
         <v>92</v>
@@ -4244,13 +4244,13 @@
         <v>0.65</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>282838</v>
+        <v>282808</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>9.097125999999999</v>
+        <v>9.096133999999999</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>8.025361</v>
+        <v>8.024487000000001</v>
       </c>
       <c r="AD28" s="2" t="n">
         <v>28.12</v>
@@ -4265,7 +4265,7 @@
         <v>12.9</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>2.3745344</v>
+        <v>2.3742757</v>
       </c>
       <c r="AI28" s="2" t="n">
         <v>481</v>
@@ -4378,13 +4378,13 @@
         <v>0.57</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>147893</v>
+        <v>148249</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>60.49542</v>
+        <v>60.64113</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>47.93509</v>
+        <v>48.05055</v>
       </c>
       <c r="AD29" s="4" t="n">
         <v>23.52</v>
@@ -4399,7 +4399,7 @@
         <v>37</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>15.483547</v>
+        <v>15.520842</v>
       </c>
       <c r="AI29" s="4" t="n">
         <v>69</v>
@@ -4512,13 +4512,13 @@
         <v>1.16</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>255211</v>
+        <v>258230</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>27.840816</v>
+        <v>28.170069</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>10.884575</v>
+        <v>11.013298</v>
       </c>
       <c r="AD30" s="2" t="n">
         <v>11.16</v>
@@ -4533,7 +4533,7 @@
         <v>125.4</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>2.6846933</v>
+        <v>2.716443</v>
       </c>
       <c r="AI30" s="2" t="n">
         <v>191</v>
@@ -4646,13 +4646,13 @@
         <v>1.3</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>277297</v>
+        <v>278786</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>14.811228</v>
+        <v>14.890711</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>14.957419</v>
+        <v>15.037688</v>
       </c>
       <c r="AD31" s="4" t="n">
         <v>16.49</v>
@@ -4667,7 +4667,7 @@
         <v>9.6</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>2.7987158</v>
+        <v>2.813735</v>
       </c>
       <c r="AI31" s="4" t="n">
         <v>410</v>
@@ -4780,13 +4780,13 @@
         <v>0.91</v>
       </c>
       <c r="AA32" s="2" t="n">
-        <v>538326</v>
+        <v>537666</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>33.48909</v>
+        <v>33.44801</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>21.284853</v>
+        <v>21.258745</v>
       </c>
       <c r="AD32" s="2" t="n">
         <v>16.95</v>
@@ -4801,7 +4801,7 @@
         <v>-34.5</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>4.925548</v>
+        <v>4.919506</v>
       </c>
       <c r="AI32" s="2" t="n">
         <v>97</v>
@@ -4914,13 +4914,13 @@
         <v>1.07</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>269083</v>
+        <v>270811</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>90.18579</v>
+        <v>90.76503</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>58.188038</v>
+        <v>58.561764</v>
       </c>
       <c r="AD33" s="4" t="n">
         <v>12.94</v>
@@ -4935,7 +4935,7 @@
         <v>19.6</v>
       </c>
       <c r="AH33" s="4" t="n">
-        <v>10.974922</v>
+        <v>11.04541</v>
       </c>
       <c r="AI33" s="4" t="n">
         <v>0</v>
@@ -5048,13 +5048,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA34" s="2" t="n">
-        <v>250254</v>
+        <v>249420</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>65.18102</v>
+        <v>64.96380000000001</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>52.11382</v>
+        <v>51.94014</v>
       </c>
       <c r="AD34" s="2" t="inlineStr"/>
       <c r="AE34" s="2" t="n">
@@ -5067,7 +5067,7 @@
         <v>-4.6</v>
       </c>
       <c r="AH34" s="2" t="n">
-        <v>12.775277</v>
+        <v>12.732701</v>
       </c>
       <c r="AI34" s="2" t="n">
         <v>96</v>
@@ -5178,13 +5178,13 @@
         <v>1.12</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>132139</v>
+        <v>133007</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>12.484921</v>
+        <v>12.5668545</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>9.53131</v>
+        <v>9.593861</v>
       </c>
       <c r="AD35" s="4" t="n">
         <v>30.41</v>
@@ -5199,7 +5199,7 @@
         <v>126.7</v>
       </c>
       <c r="AH35" s="4" t="n">
-        <v>3.70956</v>
+        <v>3.7339044</v>
       </c>
       <c r="AI35" s="4" t="n">
         <v>91</v>
@@ -5312,13 +5312,13 @@
         <v>0.5</v>
       </c>
       <c r="AA36" s="2" t="n">
-        <v>361835</v>
+        <v>364176</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>71.538055</v>
+        <v>72.00105000000001</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>47.38593</v>
+        <v>47.692608</v>
       </c>
       <c r="AD36" s="2" t="n">
         <v>37.13</v>
@@ -5333,7 +5333,7 @@
         <v>35.1</v>
       </c>
       <c r="AH36" s="2" t="n">
-        <v>28.253117</v>
+        <v>28.43597</v>
       </c>
       <c r="AI36" s="2" t="n">
         <v>27</v>
@@ -5442,13 +5442,13 @@
         <v>1.38</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>32546</v>
+        <v>32819</v>
       </c>
       <c r="AB37" s="4" t="n">
-        <v>37.483234</v>
+        <v>37.796844</v>
       </c>
       <c r="AC37" s="4" t="n">
-        <v>26.36306</v>
+        <v>26.58363</v>
       </c>
       <c r="AD37" s="4" t="inlineStr"/>
       <c r="AE37" s="4" t="n">
@@ -5461,7 +5461,7 @@
         <v>3</v>
       </c>
       <c r="AH37" s="4" t="n">
-        <v>6.072652</v>
+        <v>6.12346</v>
       </c>
       <c r="AI37" s="4" t="n">
         <v>54</v>
@@ -5572,13 +5572,13 @@
         <v>0.61</v>
       </c>
       <c r="AA38" s="2" t="n">
-        <v>140419</v>
+        <v>142086</v>
       </c>
       <c r="AB38" s="2" t="n">
-        <v>5.4196916</v>
+        <v>5.4840145</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>6.5363483</v>
+        <v>6.613924</v>
       </c>
       <c r="AD38" s="2" t="n">
         <v>20.47</v>
@@ -5593,7 +5593,7 @@
         <v>10.8</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>1.0568094</v>
+        <v>1.0693519</v>
       </c>
       <c r="AI38" s="2" t="n">
         <v>338</v>
@@ -5706,13 +5706,13 @@
         <v>1.01</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>131696</v>
+        <v>132111</v>
       </c>
       <c r="AB39" s="4" t="n">
-        <v>35.226498</v>
+        <v>35.33761</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>27.252073</v>
+        <v>27.338032</v>
       </c>
       <c r="AD39" s="4" t="n">
         <v>11.34</v>
@@ -5727,7 +5727,7 @@
         <v>-4.6</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>3.4786167</v>
+        <v>3.489589</v>
       </c>
       <c r="AI39" s="4" t="n">
         <v>60</v>
@@ -5840,13 +5840,13 @@
         <v>0.78</v>
       </c>
       <c r="AA40" s="2" t="n">
-        <v>379382</v>
+        <v>380643</v>
       </c>
       <c r="AB40" s="2" t="n">
-        <v>21.651909</v>
+        <v>21.723852</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>14.614035</v>
+        <v>14.662592</v>
       </c>
       <c r="AD40" s="2" t="inlineStr"/>
       <c r="AE40" s="2" t="n">
@@ -5859,7 +5859,7 @@
         <v>-1.6</v>
       </c>
       <c r="AH40" s="2" t="n">
-        <v>1.9738071</v>
+        <v>1.9803654</v>
       </c>
       <c r="AI40" s="2" t="n">
         <v>291</v>
@@ -5970,13 +5970,13 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>188605</v>
+        <v>188001</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>35.30061</v>
+        <v>35.187656</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>29.872179</v>
+        <v>29.776596</v>
       </c>
       <c r="AD41" s="4" t="inlineStr"/>
       <c r="AE41" s="4" t="n">
@@ -5989,7 +5989,7 @@
         <v>21.3</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>8.538278999999999</v>
+        <v>8.510959</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>102</v>
@@ -6594,13 +6594,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>138634</v>
+        <v>138476</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.072495</v>
+        <v>52.01312</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.41989</v>
+        <v>37.377224</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -6615,7 +6615,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.544624</v>
+        <v>11.531461</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -6728,13 +6728,13 @@
         <v>0.66</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>405981</v>
+        <v>408492</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>30.292248</v>
+        <v>30.47963</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>22.719347</v>
+        <v>22.859884</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>15.59</v>
@@ -6749,7 +6749,7 @@
         <v>3.6</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.2231174</v>
+        <v>4.249241</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>43</v>
@@ -6992,13 +6992,13 @@
         <v>0.77</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>108076</v>
+        <v>108711</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>61.553505</v>
+        <v>61.91513</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>44.19761</v>
+        <v>44.45727</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>41.39</v>
@@ -7013,7 +7013,7 @@
         <v>14.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>25.481182</v>
+        <v>25.630882</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>48</v>
@@ -7373,13 +7373,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>138634</v>
+        <v>138476</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.072495</v>
+        <v>52.01312</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.41989</v>
+        <v>37.377224</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -7394,7 +7394,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.544624</v>
+        <v>11.531461</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -7507,13 +7507,13 @@
         <v>0.66</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>405981</v>
+        <v>408492</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>30.292248</v>
+        <v>30.47963</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>22.719347</v>
+        <v>22.859884</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>15.59</v>
@@ -7528,7 +7528,7 @@
         <v>3.6</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.2231174</v>
+        <v>4.249241</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>43</v>
@@ -7771,13 +7771,13 @@
         <v>0.77</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>108076</v>
+        <v>108711</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>61.553505</v>
+        <v>61.91513</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>44.19761</v>
+        <v>44.45727</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>41.39</v>
@@ -7792,7 +7792,7 @@
         <v>14.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>25.481182</v>
+        <v>25.630882</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>48</v>
@@ -7837,7 +7837,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 20-May-2026 07:38 IST</t>
+          <t>Run Date: 20-May-2026 09:55 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>

</xml_diff>

<commit_message>
📈 Daily Screener Report — 20-May-2026 16:19 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -517,7 +517,7 @@
     <col width="16" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="17" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
     <col width="8" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
@@ -816,13 +816,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>138476</v>
+        <v>138491</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.01312</v>
+        <v>52.018776</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.377224</v>
+        <v>37.381287</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -837,7 +837,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.531461</v>
+        <v>11.532714</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -950,13 +950,13 @@
         <v>0.66</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>408492</v>
+        <v>408400</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>30.47963</v>
+        <v>30.472754</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>22.859884</v>
+        <v>22.854727</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>15.59</v>
@@ -971,7 +971,7 @@
         <v>3.6</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.249241</v>
+        <v>4.248282</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>43</v>
@@ -1084,13 +1084,13 @@
         <v>1.06</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>182775</v>
+        <v>182987</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>73.78631</v>
+        <v>73.87204</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>58.894444</v>
+        <v>58.962875</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="n">
@@ -1103,7 +1103,7 @@
         <v>-1</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>11.851236</v>
+        <v>11.865007</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>43</v>
@@ -1214,13 +1214,13 @@
         <v>0.77</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>108711</v>
+        <v>108647</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>61.91513</v>
+        <v>61.878227</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>44.45727</v>
+        <v>44.430775</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>41.39</v>
@@ -1235,7 +1235,7 @@
         <v>14.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>25.630882</v>
+        <v>25.615606</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>48</v>
@@ -1348,13 +1348,13 @@
         <v>0.75</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>274052</v>
+        <v>273840</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>78.17381</v>
+        <v>78.11331</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>59.993404</v>
+        <v>59.94697</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>76.34</v>
@@ -1369,7 +1369,7 @@
         <v>27.4</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>53.142876</v>
+        <v>53.101746</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>84</v>
@@ -1482,11 +1482,11 @@
         <v>0.09</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>3263</v>
+        <v>3269</v>
       </c>
       <c r="AB7" s="4" t="inlineStr"/>
       <c r="AC7" s="4" t="n">
-        <v>26.953405</v>
+        <v>27.001791</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>-2.82</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="AG7" s="4" t="inlineStr"/>
       <c r="AH7" s="4" t="n">
-        <v>5.4891715</v>
+        <v>5.499026</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>0</v>
@@ -1612,13 +1612,13 @@
         <v>0.55</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>375710</v>
+        <v>375270</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>9.875992</v>
+        <v>9.864418000000001</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>7.052684</v>
+        <v>7.0444183</v>
       </c>
       <c r="AD8" s="2" t="inlineStr"/>
       <c r="AE8" s="2" t="n">
@@ -1631,7 +1631,7 @@
         <v>16.2</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>1.0207151</v>
+        <v>1.0195189</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>624</v>
@@ -1742,13 +1742,13 @@
         <v>0.82</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>9771</v>
+        <v>9780</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>86.97978999999999</v>
+        <v>87.06303</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>44.729336</v>
+        <v>44.77214</v>
       </c>
       <c r="AD9" s="4" t="inlineStr"/>
       <c r="AE9" s="4" t="n">
@@ -1761,7 +1761,7 @@
         <v>35.8</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>14.990062</v>
+        <v>15.004406</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>0</v>
@@ -1872,13 +1872,13 @@
         <v>1.32</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>370827</v>
+        <v>370813</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>36.761345</v>
+        <v>36.75999</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>47.71809</v>
+        <v>47.716328</v>
       </c>
       <c r="AD10" s="2" t="n">
         <v>13.66</v>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="AG10" s="2" t="inlineStr"/>
       <c r="AH10" s="2" t="n">
-        <v>4.31409</v>
+        <v>4.3139305</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>5</v>
@@ -2004,13 +2004,13 @@
         <v>0.41</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>451195</v>
+        <v>451147</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>41.2843</v>
+        <v>41.279915</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>33.234688</v>
+        <v>33.23115</v>
       </c>
       <c r="AD11" s="4" t="inlineStr"/>
       <c r="AE11" s="4" t="n">
@@ -2023,7 +2023,7 @@
         <v>15.7</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>5.7957478</v>
+        <v>5.7951317</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>88</v>
@@ -2134,13 +2134,13 @@
         <v>0.61</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>313206</v>
+        <v>313182</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>14.063562</v>
+        <v>14.062466</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>17.798101</v>
+        <v>17.796713</v>
       </c>
       <c r="AD12" s="2" t="n">
         <v>27.26</v>
@@ -2155,7 +2155,7 @@
         <v>991.8</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>3.1305346</v>
+        <v>3.1302905</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>55</v>
@@ -2268,13 +2268,13 @@
         <v>1.03</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>116106</v>
+        <v>116156</v>
       </c>
       <c r="AB13" s="4" t="n">
-        <v>64.49165000000001</v>
+        <v>64.51961</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>48.528423</v>
+        <v>48.549458</v>
       </c>
       <c r="AD13" s="4" t="inlineStr"/>
       <c r="AE13" s="4" t="n">
@@ -2287,7 +2287,7 @@
         <v>35</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>12.767747</v>
+        <v>12.773281</v>
       </c>
       <c r="AI13" s="4" t="n">
         <v>25</v>
@@ -2398,13 +2398,13 @@
         <v>1.09</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>149894</v>
+        <v>149904</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>66.20179</v>
+        <v>66.206276</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>68.38627</v>
+        <v>68.39091000000001</v>
       </c>
       <c r="AD14" s="2" t="inlineStr"/>
       <c r="AE14" s="2" t="n">
@@ -2417,7 +2417,7 @@
         <v>26.1</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>17.75345</v>
+        <v>17.754654</v>
       </c>
       <c r="AI14" s="2" t="n">
         <v>78</v>
@@ -2528,13 +2528,13 @@
         <v>0.4</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>23940</v>
+        <v>23946</v>
       </c>
       <c r="AB15" s="4" t="n">
-        <v>15.54217</v>
+        <v>15.546472</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>12.619972</v>
+        <v>12.623466</v>
       </c>
       <c r="AD15" s="4" t="n">
         <v>12.55</v>
@@ -2549,7 +2549,7 @@
         <v>17.8</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>1.8811522</v>
+        <v>1.8816729</v>
       </c>
       <c r="AI15" s="4" t="n">
         <v>331</v>
@@ -2662,13 +2662,13 @@
         <v>1.24</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>87250</v>
+        <v>87314</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>25.248085</v>
+        <v>25.2664</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>19.843512</v>
+        <v>19.857904</v>
       </c>
       <c r="AD16" s="2" t="inlineStr"/>
       <c r="AE16" s="2" t="n">
@@ -2681,7 +2681,7 @@
         <v>7.6</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>2.5131133</v>
+        <v>2.5149362</v>
       </c>
       <c r="AI16" s="2" t="n">
         <v>26</v>
@@ -2792,13 +2792,13 @@
         <v>0.78</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>12671</v>
+        <v>12777</v>
       </c>
       <c r="AB17" s="4" t="n">
-        <v>30.614313</v>
+        <v>30.870806</v>
       </c>
       <c r="AC17" s="4" t="n">
-        <v>18.15019</v>
+        <v>18.302256</v>
       </c>
       <c r="AD17" s="4" t="n">
         <v>10.66</v>
@@ -2813,7 +2813,7 @@
         <v>5.9</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>3.297543</v>
+        <v>3.1557312</v>
       </c>
       <c r="AI17" s="4" t="n">
         <v>77</v>
@@ -2926,13 +2926,13 @@
         <v>0.68</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>30007</v>
+        <v>29979</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>27.303421</v>
+        <v>27.277779</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>10.877978</v>
+        <v>10.867763</v>
       </c>
       <c r="AD18" s="2" t="n">
         <v>6.97</v>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="AG18" s="2" t="inlineStr"/>
       <c r="AH18" s="2" t="n">
-        <v>1.6660582</v>
+        <v>1.6644936</v>
       </c>
       <c r="AI18" s="2" t="n">
         <v>63</v>
@@ -3058,13 +3058,13 @@
         <v>0.7</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>78417</v>
+        <v>78260</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>558.87756</v>
+        <v>557.75507</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>176.56123</v>
+        <v>176.20662</v>
       </c>
       <c r="AD19" s="4" t="inlineStr"/>
       <c r="AE19" s="4" t="n">
@@ -3077,7 +3077,7 @@
         <v>144.4</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>56.615673</v>
+        <v>56.501965</v>
       </c>
       <c r="AI19" s="4" t="n">
         <v>0</v>
@@ -3188,13 +3188,13 @@
         <v>0.42</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>20321</v>
+        <v>20324</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>23.327415</v>
+        <v>23.330967</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>17.307018</v>
+        <v>17.309652</v>
       </c>
       <c r="AD20" s="2" t="inlineStr"/>
       <c r="AE20" s="2" t="inlineStr"/>
@@ -3205,7 +3205,7 @@
         <v>367.9</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>1.2139143</v>
+        <v>1.214099</v>
       </c>
       <c r="AI20" s="2" t="n">
         <v>33</v>
@@ -3316,13 +3316,13 @@
         <v>0.37</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>59379</v>
+        <v>59285</v>
       </c>
       <c r="AB21" s="4" t="n">
-        <v>52.772022</v>
+        <v>52.68912</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>40.101646</v>
+        <v>40.03865</v>
       </c>
       <c r="AD21" s="4" t="n">
         <v>17.23</v>
@@ -3337,7 +3337,7 @@
         <v>27.7</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>8.588704</v>
+        <v>8.575212000000001</v>
       </c>
       <c r="AI21" s="4" t="n">
         <v>75</v>
@@ -3450,13 +3450,13 @@
         <v>0.46</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>19406</v>
+        <v>19340</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>59.506794</v>
+        <v>59.303013</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>35.41644</v>
+        <v>35.29516</v>
       </c>
       <c r="AD22" s="2" t="n">
         <v>14.14</v>
@@ -3471,7 +3471,7 @@
         <v>43.7</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>6.679064</v>
+        <v>6.6561913</v>
       </c>
       <c r="AI22" s="2" t="n">
         <v>15</v>
@@ -3584,13 +3584,13 @@
         <v>0.27</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>31044</v>
+        <v>30956</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>25.388668</v>
+        <v>25.316204</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>8.911617</v>
+        <v>8.886181000000001</v>
       </c>
       <c r="AD23" s="4" t="n">
         <v>4.88</v>
@@ -3603,7 +3603,7 @@
         <v>68</v>
       </c>
       <c r="AH23" s="4" t="n">
-        <v>1.2122241</v>
+        <v>1.2087642</v>
       </c>
       <c r="AI23" s="4" t="n">
         <v>78</v>
@@ -3714,13 +3714,13 @@
         <v>0.57</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>21385</v>
+        <v>21323</v>
       </c>
       <c r="AB24" s="2" t="n">
-        <v>388.19443</v>
+        <v>387.05554</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>26.875002</v>
+        <v>26.796154</v>
       </c>
       <c r="AD24" s="2" t="n">
         <v>7.27</v>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="AG24" s="2" t="inlineStr"/>
       <c r="AH24" s="2" t="n">
-        <v>4.3132715</v>
+        <v>4.3006167</v>
       </c>
       <c r="AI24" s="2" t="n">
         <v>7</v>
@@ -3846,13 +3846,13 @@
         <v>0.74</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>109944</v>
+        <v>110061</v>
       </c>
       <c r="AB25" s="4" t="n">
-        <v>26.231625</v>
+        <v>26.259436</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>20.577372</v>
+        <v>20.599188</v>
       </c>
       <c r="AD25" s="4" t="n">
         <v>11.83</v>
@@ -3867,7 +3867,7 @@
         <v>-86.2</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>2.9197161</v>
+        <v>2.9228117</v>
       </c>
       <c r="AI25" s="4" t="n">
         <v>60</v>
@@ -3980,13 +3980,13 @@
         <v>0.86</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>71470</v>
+        <v>71434</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>16.593248</v>
+        <v>16.58467</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>12.207583</v>
+        <v>12.20127</v>
       </c>
       <c r="AD26" s="2" t="n">
         <v>11.73</v>
@@ -3999,7 +3999,7 @@
         <v>22.2</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>1.9637114</v>
+        <v>1.9626958</v>
       </c>
       <c r="AI26" s="2" t="n">
         <v>42</v>
@@ -4110,13 +4110,13 @@
         <v>0.61</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>112987</v>
+        <v>113052</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>29.18214</v>
+        <v>29.198832</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>22.079332</v>
+        <v>22.091963</v>
       </c>
       <c r="AD27" s="4" t="n">
         <v>11.74</v>
@@ -4131,7 +4131,7 @@
         <v>-54.6</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>3.4321313</v>
+        <v>3.4340944</v>
       </c>
       <c r="AI27" s="4" t="n">
         <v>92</v>
@@ -4244,13 +4244,13 @@
         <v>0.65</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>282808</v>
+        <v>282684</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>9.096133999999999</v>
+        <v>9.092171</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>8.024487000000001</v>
+        <v>8.020989</v>
       </c>
       <c r="AD28" s="2" t="n">
         <v>28.12</v>
@@ -4265,7 +4265,7 @@
         <v>12.9</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>2.3742757</v>
+        <v>2.373241</v>
       </c>
       <c r="AI28" s="2" t="n">
         <v>481</v>
@@ -4378,13 +4378,13 @@
         <v>0.57</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>148249</v>
+        <v>148147</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>60.64113</v>
+        <v>60.5995</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>48.05055</v>
+        <v>48.01756</v>
       </c>
       <c r="AD29" s="4" t="n">
         <v>23.52</v>
@@ -4399,7 +4399,7 @@
         <v>37</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>15.520842</v>
+        <v>15.510186</v>
       </c>
       <c r="AI29" s="4" t="n">
         <v>69</v>
@@ -4512,13 +4512,13 @@
         <v>1.16</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>258230</v>
+        <v>258180</v>
       </c>
       <c r="AB30" s="2" t="n">
-        <v>28.170069</v>
+        <v>28.164625</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>11.013298</v>
+        <v>11.01117</v>
       </c>
       <c r="AD30" s="2" t="n">
         <v>11.16</v>
@@ -4533,7 +4533,7 @@
         <v>125.4</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>2.716443</v>
+        <v>2.715918</v>
       </c>
       <c r="AI30" s="2" t="n">
         <v>191</v>
@@ -4646,13 +4646,13 @@
         <v>1.3</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>278786</v>
+        <v>278925</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>14.890711</v>
+        <v>14.898162</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>15.037688</v>
+        <v>15.045213</v>
       </c>
       <c r="AD31" s="4" t="n">
         <v>16.49</v>
@@ -4667,7 +4667,7 @@
         <v>9.6</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>2.813735</v>
+        <v>2.815143</v>
       </c>
       <c r="AI31" s="4" t="n">
         <v>410</v>
@@ -4780,13 +4780,13 @@
         <v>0.91</v>
       </c>
       <c r="AA32" s="2" t="n">
-        <v>537666</v>
+        <v>537983</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>33.44801</v>
+        <v>33.467693</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>21.258745</v>
+        <v>21.271255</v>
       </c>
       <c r="AD32" s="2" t="n">
         <v>16.95</v>
@@ -4801,7 +4801,7 @@
         <v>-34.5</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>4.919506</v>
+        <v>4.9224014</v>
       </c>
       <c r="AI32" s="2" t="n">
         <v>97</v>
@@ -4914,13 +4914,13 @@
         <v>1.07</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>270811</v>
+        <v>270270</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>90.76503</v>
+        <v>90.58360999999999</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>58.561764</v>
+        <v>58.444714</v>
       </c>
       <c r="AD33" s="4" t="n">
         <v>12.94</v>
@@ -4935,7 +4935,7 @@
         <v>19.6</v>
       </c>
       <c r="AH33" s="4" t="n">
-        <v>11.04541</v>
+        <v>11.023334</v>
       </c>
       <c r="AI33" s="4" t="n">
         <v>0</v>
@@ -5048,13 +5048,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA34" s="2" t="n">
-        <v>249420</v>
+        <v>249113</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>64.96380000000001</v>
+        <v>64.88389599999999</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>51.94014</v>
+        <v>51.87626</v>
       </c>
       <c r="AD34" s="2" t="inlineStr"/>
       <c r="AE34" s="2" t="n">
@@ -5067,7 +5067,7 @@
         <v>-4.6</v>
       </c>
       <c r="AH34" s="2" t="n">
-        <v>12.732701</v>
+        <v>12.717041</v>
       </c>
       <c r="AI34" s="2" t="n">
         <v>96</v>
@@ -5178,13 +5178,13 @@
         <v>1.12</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>133007</v>
+        <v>132858</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>12.5668545</v>
+        <v>12.55282</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>9.593861</v>
+        <v>9.583145999999999</v>
       </c>
       <c r="AD35" s="4" t="n">
         <v>30.41</v>
@@ -5199,7 +5199,7 @@
         <v>126.7</v>
       </c>
       <c r="AH35" s="4" t="n">
-        <v>3.7339044</v>
+        <v>3.7297342</v>
       </c>
       <c r="AI35" s="4" t="n">
         <v>91</v>
@@ -5312,13 +5312,13 @@
         <v>0.5</v>
       </c>
       <c r="AA36" s="2" t="n">
-        <v>364176</v>
+        <v>364256</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>72.00105000000001</v>
+        <v>72.01683</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>47.692608</v>
+        <v>47.703064</v>
       </c>
       <c r="AD36" s="2" t="n">
         <v>37.13</v>
@@ -5333,7 +5333,7 @@
         <v>35.1</v>
       </c>
       <c r="AH36" s="2" t="n">
-        <v>28.43597</v>
+        <v>28.442204</v>
       </c>
       <c r="AI36" s="2" t="n">
         <v>27</v>
@@ -5442,13 +5442,13 @@
         <v>1.38</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>32819</v>
+        <v>32833</v>
       </c>
       <c r="AB37" s="4" t="n">
-        <v>37.796844</v>
+        <v>37.812622</v>
       </c>
       <c r="AC37" s="4" t="n">
-        <v>26.58363</v>
+        <v>26.594727</v>
       </c>
       <c r="AD37" s="4" t="inlineStr"/>
       <c r="AE37" s="4" t="n">
@@ -5461,7 +5461,7 @@
         <v>3</v>
       </c>
       <c r="AH37" s="4" t="n">
-        <v>6.12346</v>
+        <v>6.126016</v>
       </c>
       <c r="AI37" s="4" t="n">
         <v>54</v>
@@ -5572,13 +5572,13 @@
         <v>0.61</v>
       </c>
       <c r="AA38" s="2" t="n">
-        <v>142086</v>
+        <v>141690</v>
       </c>
       <c r="AB38" s="2" t="n">
-        <v>5.4840145</v>
+        <v>5.46873</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>6.613924</v>
+        <v>6.5954905</v>
       </c>
       <c r="AD38" s="2" t="n">
         <v>20.47</v>
@@ -5593,7 +5593,7 @@
         <v>10.8</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>1.0693519</v>
+        <v>1.0663716</v>
       </c>
       <c r="AI38" s="2" t="n">
         <v>338</v>
@@ -5706,13 +5706,13 @@
         <v>1.01</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>132111</v>
+        <v>132127</v>
       </c>
       <c r="AB39" s="4" t="n">
-        <v>35.33761</v>
+        <v>35.34188</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>27.338032</v>
+        <v>27.341337</v>
       </c>
       <c r="AD39" s="4" t="n">
         <v>11.34</v>
@@ -5727,7 +5727,7 @@
         <v>-4.6</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>3.489589</v>
+        <v>3.490011</v>
       </c>
       <c r="AI39" s="4" t="n">
         <v>60</v>
@@ -5840,13 +5840,13 @@
         <v>0.78</v>
       </c>
       <c r="AA40" s="2" t="n">
-        <v>380643</v>
+        <v>380546</v>
       </c>
       <c r="AB40" s="2" t="n">
-        <v>21.723852</v>
+        <v>21.718319</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>14.662592</v>
+        <v>14.658858</v>
       </c>
       <c r="AD40" s="2" t="inlineStr"/>
       <c r="AE40" s="2" t="n">
@@ -5859,7 +5859,7 @@
         <v>-1.6</v>
       </c>
       <c r="AH40" s="2" t="n">
-        <v>1.9803654</v>
+        <v>1.979861</v>
       </c>
       <c r="AI40" s="2" t="n">
         <v>291</v>
@@ -5970,13 +5970,13 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>188001</v>
+        <v>187892</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>35.187656</v>
+        <v>35.167118</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>29.776596</v>
+        <v>29.759216</v>
       </c>
       <c r="AD41" s="4" t="inlineStr"/>
       <c r="AE41" s="4" t="n">
@@ -5989,7 +5989,7 @@
         <v>21.3</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>8.510959</v>
+        <v>8.505991</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>102</v>
@@ -6594,13 +6594,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>138476</v>
+        <v>138491</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.01312</v>
+        <v>52.018776</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.377224</v>
+        <v>37.381287</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -6615,7 +6615,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.531461</v>
+        <v>11.532714</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -6728,13 +6728,13 @@
         <v>0.66</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>408492</v>
+        <v>408400</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>30.47963</v>
+        <v>30.472754</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>22.859884</v>
+        <v>22.854727</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>15.59</v>
@@ -6749,7 +6749,7 @@
         <v>3.6</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.249241</v>
+        <v>4.248282</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>43</v>
@@ -6862,13 +6862,13 @@
         <v>1.06</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>182775</v>
+        <v>182987</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>73.78631</v>
+        <v>73.87204</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>58.894444</v>
+        <v>58.962875</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="n">
@@ -6881,7 +6881,7 @@
         <v>-1</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>11.851236</v>
+        <v>11.865007</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>43</v>
@@ -6992,13 +6992,13 @@
         <v>0.77</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>108711</v>
+        <v>108647</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>61.91513</v>
+        <v>61.878227</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>44.45727</v>
+        <v>44.430775</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>41.39</v>
@@ -7013,7 +7013,7 @@
         <v>14.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>25.630882</v>
+        <v>25.615606</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>48</v>
@@ -7373,13 +7373,13 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>138476</v>
+        <v>138491</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>52.01312</v>
+        <v>52.018776</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>37.377224</v>
+        <v>37.381287</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>24.58</v>
@@ -7394,7 +7394,7 @@
         <v>8</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>11.531461</v>
+        <v>11.532714</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>38</v>
@@ -7507,13 +7507,13 @@
         <v>0.66</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>408492</v>
+        <v>408400</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>30.47963</v>
+        <v>30.472754</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>22.859884</v>
+        <v>22.854727</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>15.59</v>
@@ -7528,7 +7528,7 @@
         <v>3.6</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>4.249241</v>
+        <v>4.248282</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>43</v>
@@ -7641,13 +7641,13 @@
         <v>1.06</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>182775</v>
+        <v>182987</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>73.78631</v>
+        <v>73.87204</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>58.894444</v>
+        <v>58.962875</v>
       </c>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="n">
@@ -7660,7 +7660,7 @@
         <v>-1</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>11.851236</v>
+        <v>11.865007</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>43</v>
@@ -7771,13 +7771,13 @@
         <v>0.77</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>108711</v>
+        <v>108647</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>61.91513</v>
+        <v>61.878227</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>44.45727</v>
+        <v>44.430775</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>41.39</v>
@@ -7792,7 +7792,7 @@
         <v>14.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>25.630882</v>
+        <v>25.615606</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>48</v>
@@ -7837,7 +7837,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 20-May-2026 09:55 IST</t>
+          <t>Run Date: 20-May-2026 10:49 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>

</xml_diff>

<commit_message>
📈 Daily Screener Report — 21-May-2026 00:14 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -2534,7 +2534,7 @@
         <v>15.546472</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>12.623466</v>
+        <v>12.598603</v>
       </c>
       <c r="AD15" s="4" t="n">
         <v>12.55</v>
@@ -2813,7 +2813,7 @@
         <v>5.9</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>3.1557312</v>
+        <v>3.3251705</v>
       </c>
       <c r="AI17" s="4" t="n">
         <v>77</v>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="AG24" s="2" t="inlineStr"/>
       <c r="AH24" s="2" t="n">
-        <v>4.3006167</v>
+        <v>4.2029376</v>
       </c>
       <c r="AI24" s="2" t="n">
         <v>7</v>
@@ -3852,7 +3852,7 @@
         <v>26.259436</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>20.599188</v>
+        <v>20.629068</v>
       </c>
       <c r="AD25" s="4" t="n">
         <v>11.83</v>
@@ -4652,7 +4652,7 @@
         <v>14.898162</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>15.045213</v>
+        <v>15.056037</v>
       </c>
       <c r="AD31" s="4" t="n">
         <v>16.49</v>
@@ -7837,7 +7837,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 20-May-2026 10:49 IST</t>
+          <t>Run Date: 20-May-2026 18:44 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>

</xml_diff>

<commit_message>
📈 Daily Screener Report — 30-May-2026 00:13 IST
</commit_message>
<xml_diff>
--- a/output/swing_screener_report.xlsx
+++ b/output/swing_screener_report.xlsx
@@ -775,7 +775,7 @@
         <v>324.82</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>296.89</v>
+        <v>296.83</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -816,13 +816,13 @@
         <v>1.01</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>21540</v>
+        <v>21360</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>24.673758</v>
+        <v>24.468084</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>18.331898</v>
+        <v>18.179089</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -833,7 +833,7 @@
         <v>367.9</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>1.2857991</v>
+        <v>1.2750812</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>33</v>
@@ -903,7 +903,7 @@
         <v>453.89</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>417.78</v>
+        <v>417.31</v>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
@@ -944,13 +944,13 @@
         <v>7.74</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>285704</v>
+        <v>282191</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>9.185655000000001</v>
+        <v>9.072716</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>8.106672</v>
+        <v>8.007</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>28.12</v>
@@ -965,7 +965,7 @@
         <v>12.9</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>2.3985927</v>
+        <v>2.3691018</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>475</v>
@@ -1037,7 +1037,7 @@
         <v>1641.65</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1490.46</v>
+        <v>1490.49</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -1078,13 +1078,13 @@
         <v>0.66</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>420012</v>
+        <v>415772</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>31.323023</v>
+        <v>31.006872</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>23.50455</v>
+        <v>23.267313</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>15.59</v>
@@ -1099,7 +1099,7 @@
         <v>3.6</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>4.369073</v>
+        <v>4.3249745</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>41</v>
@@ -1171,7 +1171,7 @@
         <v>6510.26</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>6303.62</v>
+        <v>6303.55</v>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
@@ -1212,13 +1212,13 @@
         <v>0.43</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>180280</v>
+        <v>176988</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>70.358475</v>
+        <v>69.07377</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>48.03056</v>
+        <v>47.15355</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>16.19</v>
@@ -1233,7 +1233,7 @@
         <v>13.6</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>11.689433</v>
+        <v>11.47599</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>44</v>
@@ -1305,7 +1305,7 @@
         <v>1189.85</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>1017.63</v>
+        <v>1017.19</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -1346,13 +1346,13 @@
         <v>0.35</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>9965</v>
+        <v>10155</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>88.17967</v>
+        <v>89.86407</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>45.615974</v>
+        <v>46.487324</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>16.94</v>
@@ -1367,7 +1367,7 @@
         <v>69</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>13.810468</v>
+        <v>14.074273</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>0</v>
@@ -1439,7 +1439,7 @@
         <v>8441.25</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>7560.62</v>
+        <v>7561.76</v>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
@@ -1480,13 +1480,13 @@
         <v>0.49</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>145462</v>
+        <v>142684</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>54.63387</v>
+        <v>53.59061</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>39.262745</v>
+        <v>38.51301</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>24.58</v>
@@ -1501,7 +1501,7 @@
         <v>8</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>12.1131735</v>
+        <v>11.881867</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>36</v>
@@ -1573,7 +1573,7 @@
         <v>7830.53</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>7493.93</v>
+        <v>7498.69</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -1614,13 +1614,13 @@
         <v>0.67</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>119047</v>
+        <v>117566</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>61.402405</v>
+        <v>60.638535</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>38.752354</v>
+        <v>38.27026</v>
       </c>
       <c r="AD8" s="2" t="n">
         <v>21.5</v>
@@ -1635,7 +1635,7 @@
         <v>35.6</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>12.554779</v>
+        <v>12.398593</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>24</v>
@@ -1707,7 +1707,7 @@
         <v>4296.48</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>3957.95</v>
+        <v>3950.73</v>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
@@ -1748,13 +1748,13 @@
         <v>0.7</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>153285</v>
+        <v>149282</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>70.789314</v>
+        <v>68.94029</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>47.70262</v>
+        <v>46.456627</v>
       </c>
       <c r="AD9" s="4" t="n">
         <v>16.98</v>
@@ -1769,7 +1769,7 @@
         <v>-21.8</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>18.155107</v>
+        <v>17.680895</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>84</v>
@@ -1841,7 +1841,7 @@
         <v>1249.42</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1171.93</v>
+        <v>1171.38</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1882,13 +1882,13 @@
         <v>1.14</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>319723</v>
+        <v>311913</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>14.354591</v>
+        <v>14.003944</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>18.041344</v>
+        <v>17.60064</v>
       </c>
       <c r="AD10" s="2" t="n">
         <v>27.26</v>
@@ -1903,7 +1903,7 @@
         <v>991.8</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>3.1956675</v>
+        <v>3.1176054</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>54</v>
@@ -1975,7 +1975,7 @@
         <v>415.21</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>360.58</v>
+        <v>360.33</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -2016,13 +2016,13 @@
         <v>0.16</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>12713</v>
+        <v>12407</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>30.676786</v>
+        <v>29.93991</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>18.210266</v>
+        <v>17.772844</v>
       </c>
       <c r="AD11" s="4" t="n">
         <v>10.66</v>
@@ -2037,7 +2037,7 @@
         <v>-85.59999999999999</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>3.13987</v>
+        <v>22.567343</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>77</v>
@@ -2109,7 +2109,7 @@
         <v>174.62</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>165.04</v>
+        <v>165.02</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -2150,13 +2150,13 @@
         <v>0.98</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>24698</v>
+        <v>24137</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>16.006872</v>
+        <v>15.64347</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>12.994033</v>
+        <v>12.69903</v>
       </c>
       <c r="AD12" s="2" t="n">
         <v>12.55</v>
@@ -2171,7 +2171,7 @@
         <v>17.8</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>1.9407324</v>
+        <v>1.896672</v>
       </c>
       <c r="AI12" s="2" t="n">
         <v>323</v>
@@ -2243,7 +2243,7 @@
         <v>1373.82</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>1280.08</v>
+        <v>1282.17</v>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
@@ -2284,13 +2284,13 @@
         <v>0.66</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>275286</v>
+        <v>274110</v>
       </c>
       <c r="AB13" s="4" t="n">
-        <v>78.74242</v>
+        <v>78.40595999999999</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>60.26357</v>
+        <v>60.00607</v>
       </c>
       <c r="AD13" s="4" t="n">
         <v>76.34</v>
@@ -2305,7 +2305,7 @@
         <v>27.4</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>53.38219</v>
+        <v>53.154095</v>
       </c>
       <c r="AI13" s="4" t="n">
         <v>84</v>
@@ -2377,7 +2377,7 @@
         <v>796.6</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>754.84</v>
+        <v>755.76</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -2418,13 +2418,13 @@
         <v>0.53</v>
       </c>
       <c r="AA14" s="2" t="n">
-        <v>108329</v>
+        <v>106477</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>61.51582</v>
+        <v>60.463577</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>44.300945</v>
+        <v>43.543167</v>
       </c>
       <c r="AD14" s="2" t="n">
         <v>41.39</v>
@@ -2439,7 +2439,7 @@
         <v>14.5</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>25.540756</v>
+        <v>25.103876</v>
       </c>
       <c r="AI14" s="2" t="n">
         <v>48</v>
@@ -2511,7 +2511,7 @@
         <v>955.88</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>810.47</v>
+        <v>810.38</v>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
@@ -2552,13 +2552,13 @@
         <v>0.31</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>20322</v>
+        <v>20968</v>
       </c>
       <c r="AB15" s="4" t="n">
-        <v>62.168533</v>
+        <v>64.14555</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>37.08804</v>
+        <v>38.267475</v>
       </c>
       <c r="AD15" s="4" t="n">
         <v>14.14</v>
@@ -2573,7 +2573,7 @@
         <v>43.7</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>6.9943047</v>
+        <v>7.2167306</v>
       </c>
       <c r="AI15" s="4" t="n">
         <v>14</v>
@@ -2645,7 +2645,7 @@
         <v>3915.91</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>3812.51</v>
+        <v>3806.13</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -2686,13 +2686,13 @@
         <v>0.66</v>
       </c>
       <c r="AA16" s="2" t="n">
-        <v>557146</v>
+        <v>560791</v>
       </c>
       <c r="AB16" s="2" t="n">
-        <v>34.624264</v>
+        <v>34.850815</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>22.066845</v>
+        <v>22.211233</v>
       </c>
       <c r="AD16" s="2" t="n">
         <v>16.95</v>
@@ -2707,7 +2707,7 @@
         <v>-34.5</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>5.0977383</v>
+        <v>5.131094</v>
       </c>
       <c r="AI16" s="2" t="n">
         <v>94</v>
@@ -2779,7 +2779,7 @@
         <v>2420.31</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>2303.67</v>
+        <v>2300.71</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
@@ -2820,13 +2820,13 @@
         <v>1.27</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>407554</v>
+        <v>402701</v>
       </c>
       <c r="AB17" s="4" t="n">
-        <v>40.320087</v>
+        <v>39.839954</v>
       </c>
       <c r="AC17" s="4" t="n">
-        <v>52.44421</v>
+        <v>51.819702</v>
       </c>
       <c r="AD17" s="4" t="n">
         <v>13.66</v>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="AG17" s="4" t="inlineStr"/>
       <c r="AH17" s="4" t="n">
-        <v>4.7413683</v>
+        <v>4.684908</v>
       </c>
       <c r="AI17" s="4" t="n">
         <v>4</v>
@@ -2911,7 +2911,7 @@
         <v>184.53</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>168.23</v>
+        <v>168.04</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -2952,13 +2952,13 @@
         <v>1.04</v>
       </c>
       <c r="AA18" s="2" t="n">
-        <v>33187</v>
+        <v>33558</v>
       </c>
       <c r="AB18" s="2" t="n">
-        <v>27.105263</v>
+        <v>27.407896</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>9.550098</v>
+        <v>9.656726000000001</v>
       </c>
       <c r="AD18" s="2" t="n">
         <v>4.88</v>
@@ -2971,7 +2971,7 @@
         <v>68</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>1.2958908</v>
+        <v>1.3103596</v>
       </c>
       <c r="AI18" s="2" t="n">
         <v>73</v>
@@ -3041,7 +3041,7 @@
         <v>387.53</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>360.81</v>
+        <v>360.6</v>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
@@ -3082,13 +3082,13 @@
         <v>1.7</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>385782</v>
+        <v>375164</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>13.061393</v>
+        <v>12.701904</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>14.062249</v>
+        <v>13.675214</v>
       </c>
       <c r="AD19" s="4" t="n">
         <v>13.69</v>
@@ -3103,7 +3103,7 @@
         <v>-1.6</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>1.8995532</v>
+        <v>1.8472718</v>
       </c>
       <c r="AI19" s="4" t="n">
         <v>285</v>
@@ -3175,7 +3175,7 @@
         <v>297.17</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>281.61</v>
+        <v>281.36</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -3216,13 +3216,13 @@
         <v>0.37</v>
       </c>
       <c r="AA20" s="2" t="n">
-        <v>30904</v>
+        <v>30566</v>
       </c>
       <c r="AB20" s="2" t="n">
-        <v>28.11966</v>
+        <v>27.811966</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>11.2031765</v>
+        <v>11.080588</v>
       </c>
       <c r="AD20" s="2" t="n">
         <v>6.97</v>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="AG20" s="2" t="inlineStr"/>
       <c r="AH20" s="2" t="n">
-        <v>1.7158651</v>
+        <v>1.6970897</v>
       </c>
       <c r="AI20" s="2" t="n">
         <v>61</v>
@@ -3303,7 +3303,7 @@
         <v>1285.23</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>1250.1</v>
+        <v>1249.12</v>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
@@ -3344,13 +3344,13 @@
         <v>1.07</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>405691</v>
+        <v>400124</v>
       </c>
       <c r="AB21" s="4" t="n">
-        <v>15.436043</v>
+        <v>15.224233</v>
       </c>
       <c r="AC21" s="4" t="n">
-        <v>10.353174</v>
+        <v>10.211111</v>
       </c>
       <c r="AD21" s="4" t="n">
         <v>13.15</v>
@@ -3363,7 +3363,7 @@
         <v>6.4</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>1.8847942</v>
+        <v>1.8589315</v>
       </c>
       <c r="AI21" s="4" t="n">
         <v>8</v>
@@ -3383,12 +3383,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>UNIONBANK</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Canara Bank</t>
+          <t>Union Bank of India</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3405,10 +3405,10 @@
         <v>53.9</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>25.5</v>
+        <v>28.5</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>28.4</v>
+        <v>25.4</v>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
@@ -3417,19 +3417,19 @@
       </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n">
-        <v>134.16</v>
+        <v>168.72</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0.76</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>132</v>
+        <v>166.16</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>135.46</v>
+        <v>170.92</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>133</v>
+        <v>161.51</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -3442,120 +3442,120 @@
         </is>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>82.36</v>
+        <v>82.11</v>
       </c>
       <c r="R22" s="2" t="n">
-        <v>52.71</v>
+        <v>51.67</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>-1.5506</v>
+        <v>-2.6548</v>
       </c>
       <c r="T22" s="2" t="n">
-        <v>-2.2398</v>
+        <v>-3.9353</v>
       </c>
       <c r="U22" s="2" t="n">
-        <v>0.6892</v>
+        <v>1.2805</v>
       </c>
       <c r="V22" s="2" t="inlineStr"/>
       <c r="W22" s="2" t="n">
-        <v>14.83</v>
+        <v>20.05</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>26115218</v>
+        <v>7569728</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>23758342</v>
+        <v>11278254</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>1.1</v>
+        <v>0.67</v>
       </c>
       <c r="AA22" s="2" t="n">
-        <v>121819</v>
+        <v>128153</v>
       </c>
       <c r="AB22" s="2" t="n">
-        <v>6.180396</v>
+        <v>6.5990567</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>5.813008</v>
+        <v>6.5414696</v>
       </c>
       <c r="AD22" s="2" t="n">
-        <v>17.57</v>
+        <v>15.71</v>
       </c>
       <c r="AE22" s="2" t="inlineStr"/>
-      <c r="AF22" s="2" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="AG22" s="2" t="n">
-        <v>-9.800000000000001</v>
-      </c>
+      <c r="AF22" s="2" t="inlineStr"/>
+      <c r="AG22" s="2" t="inlineStr"/>
       <c r="AH22" s="2" t="n">
-        <v>1.0355463</v>
+        <v>0.9779855</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>313</v>
+        <v>282</v>
       </c>
       <c r="AJ22" s="2" t="inlineStr"/>
       <c r="AK22" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/CANBK/</t>
+          <t>https://www.screener.in/company/UNIONBANK/</t>
         </is>
       </c>
       <c r="AL22" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:CANBK</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:UNIONBANK</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>UNIONBANK</t>
+          <t>WAAREEENER</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Union Bank of India</t>
+          <t>WAAREEENER</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Banks - Regional</t>
+          <t>Solar</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>53.9</v>
+        <v>52.4</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>28.5</v>
+        <v>24</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>25.4</v>
+        <v>28.4</v>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>💎 High ROE</t>
+        </is>
+      </c>
       <c r="J23" s="4" t="n">
-        <v>168.72</v>
+        <v>3129.1</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.33</v>
       </c>
       <c r="L23" s="4" t="n">
-        <v>166.16</v>
+        <v>3106.94</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>170.92</v>
+        <v>3114.39</v>
       </c>
       <c r="N23" s="4" t="n">
-        <v>161.75</v>
+        <v>3015.33</v>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
@@ -3568,95 +3568,103 @@
         </is>
       </c>
       <c r="Q23" s="4" t="n">
-        <v>82.11</v>
+        <v>81.01000000000001</v>
       </c>
       <c r="R23" s="4" t="n">
-        <v>51.67</v>
+        <v>50.67</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>-2.6548</v>
+        <v>-44.04</v>
       </c>
       <c r="T23" s="4" t="n">
-        <v>-3.9353</v>
+        <v>-41.3219</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>1.2805</v>
+        <v>-2.7181</v>
       </c>
       <c r="V23" s="4" t="inlineStr"/>
       <c r="W23" s="4" t="n">
-        <v>20.05</v>
+        <v>15.59</v>
       </c>
       <c r="X23" s="4" t="n">
-        <v>7569728</v>
+        <v>1978239</v>
       </c>
       <c r="Y23" s="4" t="n">
-        <v>11278254</v>
+        <v>1420556</v>
       </c>
       <c r="Z23" s="4" t="n">
-        <v>0.67</v>
+        <v>1.39</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>128817</v>
+        <v>90346</v>
       </c>
       <c r="AB23" s="4" t="n">
-        <v>6.6332545</v>
+        <v>27.650322</v>
       </c>
       <c r="AC23" s="4" t="n">
-        <v>6.575369</v>
+        <v>18.104729</v>
       </c>
       <c r="AD23" s="4" t="n">
-        <v>15.71</v>
-      </c>
-      <c r="AE23" s="4" t="inlineStr"/>
-      <c r="AF23" s="4" t="inlineStr"/>
-      <c r="AG23" s="4" t="inlineStr"/>
+        <v>31.57</v>
+      </c>
+      <c r="AE23" s="4" t="n">
+        <v>21.402</v>
+      </c>
+      <c r="AF23" s="4" t="n">
+        <v>111.8</v>
+      </c>
+      <c r="AG23" s="4" t="n">
+        <v>71.2</v>
+      </c>
       <c r="AH23" s="4" t="n">
-        <v>0.9830536</v>
+        <v>6.254107</v>
       </c>
       <c r="AI23" s="4" t="n">
-        <v>282</v>
-      </c>
-      <c r="AJ23" s="4" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="AJ23" s="4" t="n">
+        <v>1.383</v>
+      </c>
       <c r="AK23" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/UNIONBANK/</t>
+          <t>https://www.screener.in/company/WAAREEENER/</t>
         </is>
       </c>
       <c r="AL23" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:UNIONBANK</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:WAAREEENER</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>WAAREEENER</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>WAAREEENER</t>
+          <t>Eicher Motors Limited</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Solar</t>
+          <t>Auto Manufacturers</t>
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>52.4</v>
+        <v>52.2</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>28.4</v>
+        <v>22.2</v>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
@@ -3665,23 +3673,23 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>💎 High ROE</t>
+          <t>✅ Supertrend Buy | 💎 High ROE</t>
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>3129.1</v>
+        <v>7419</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>1.33</v>
+        <v>0.58</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>3106.94</v>
+        <v>7140.39</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>3114.39</v>
+        <v>7153</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3013.23</v>
+        <v>6893.68</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -3690,107 +3698,107 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>81.01000000000001</v>
+        <v>90.15000000000001</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>50.67</v>
+        <v>61.37</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>-44.04</v>
+        <v>25.8987</v>
       </c>
       <c r="T24" s="2" t="n">
-        <v>-41.3219</v>
+        <v>-13.9708</v>
       </c>
       <c r="U24" s="2" t="n">
-        <v>-2.7181</v>
+        <v>39.8696</v>
       </c>
       <c r="V24" s="2" t="inlineStr"/>
       <c r="W24" s="2" t="n">
-        <v>15.59</v>
+        <v>16.72</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>1978239</v>
+        <v>283327</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>1420556</v>
+        <v>464892</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>1.39</v>
+        <v>0.61</v>
       </c>
       <c r="AA24" s="2" t="n">
-        <v>90466</v>
+        <v>197007</v>
       </c>
       <c r="AB24" s="2" t="n">
-        <v>27.687298</v>
+        <v>35.697586</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>18.128939</v>
+        <v>27.068094</v>
       </c>
       <c r="AD24" s="2" t="n">
-        <v>31.57</v>
+        <v>23.77</v>
       </c>
       <c r="AE24" s="2" t="n">
-        <v>21.402</v>
+        <v>2.048</v>
       </c>
       <c r="AF24" s="2" t="n">
-        <v>111.8</v>
+        <v>19.1</v>
       </c>
       <c r="AG24" s="2" t="n">
-        <v>71.2</v>
+        <v>11.5</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>6.2624702</v>
+        <v>7.8434587</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>13</v>
+        <v>94</v>
       </c>
       <c r="AJ24" s="2" t="n">
-        <v>1.383</v>
+        <v>1.902</v>
       </c>
       <c r="AK24" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/WAAREEENER/</t>
+          <t>https://www.screener.in/company/EICHERMOT/</t>
         </is>
       </c>
       <c r="AL24" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:WAAREEENER</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:EICHERMOT</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Eicher Motors Limited</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Auto Manufacturers</t>
+          <t>Drug Manufacturers - Specialty &amp; Generic</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>52.2</v>
+        <v>51.6</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>22.2</v>
+        <v>18.6</v>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
@@ -3799,27 +3807,27 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 💎 High ROE</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High</t>
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>7419</v>
+        <v>1844.3</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>0.58</v>
+        <v>0.19</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>7140.39</v>
+        <v>1836.01</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>7153</v>
+        <v>1793.25</v>
       </c>
       <c r="N25" s="4" t="n">
-        <v>6892.06</v>
+        <v>1728.73</v>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="P25" s="4" t="inlineStr">
@@ -3828,103 +3836,103 @@
         </is>
       </c>
       <c r="Q25" s="4" t="n">
-        <v>90.15000000000001</v>
+        <v>96.23</v>
       </c>
       <c r="R25" s="4" t="n">
-        <v>61.37</v>
+        <v>54.45</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>25.8987</v>
+        <v>26.3583</v>
       </c>
       <c r="T25" s="4" t="n">
-        <v>-13.9708</v>
+        <v>32.6871</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>39.8696</v>
+        <v>-6.3288</v>
       </c>
       <c r="V25" s="4" t="inlineStr"/>
       <c r="W25" s="4" t="n">
-        <v>16.72</v>
+        <v>25.63</v>
       </c>
       <c r="X25" s="4" t="n">
-        <v>283327</v>
+        <v>1385752</v>
       </c>
       <c r="Y25" s="4" t="n">
-        <v>464892</v>
+        <v>2613156</v>
       </c>
       <c r="Z25" s="4" t="n">
-        <v>0.61</v>
+        <v>0.53</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>203842</v>
+        <v>431688</v>
       </c>
       <c r="AB25" s="4" t="n">
-        <v>36.936085</v>
+        <v>37.663803</v>
       </c>
       <c r="AC25" s="4" t="n">
-        <v>28.007198</v>
+        <v>27.768585</v>
       </c>
       <c r="AD25" s="4" t="n">
-        <v>23.77</v>
+        <v>14.72</v>
       </c>
       <c r="AE25" s="4" t="n">
-        <v>2.048</v>
+        <v>5.517</v>
       </c>
       <c r="AF25" s="4" t="n">
-        <v>19.1</v>
+        <v>12.8</v>
       </c>
       <c r="AG25" s="4" t="n">
-        <v>11.5</v>
+        <v>25.6</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>8.115581000000001</v>
+        <v>5.5451794</v>
       </c>
       <c r="AI25" s="4" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>1.902</v>
+        <v>2.824</v>
       </c>
       <c r="AK25" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/EICHERMOT/</t>
+          <t>https://www.screener.in/company/SUNPHARMA/</t>
         </is>
       </c>
       <c r="AL25" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:EICHERMOT</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:SUNPHARMA</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>FEDERALBNK</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>The Federal Bank Limited</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Drug Manufacturers - Specialty &amp; Generic</t>
+          <t>Banks - Regional</t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>51.6</v>
+        <v>50.6</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>18.6</v>
+        <v>23.6</v>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
@@ -3937,19 +3945,19 @@
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>1844.3</v>
+        <v>288.9</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0.19</v>
+        <v>-0.45</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>1836.01</v>
+        <v>287.49</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>1793.25</v>
+        <v>284.75</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1730.9</v>
+        <v>258.6</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -3962,103 +3970,99 @@
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>96.23</v>
+        <v>95.66</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>54.45</v>
+        <v>52.42</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>26.3583</v>
+        <v>0.5874</v>
       </c>
       <c r="T26" s="2" t="n">
-        <v>32.6871</v>
+        <v>0.6284</v>
       </c>
       <c r="U26" s="2" t="n">
-        <v>-6.3288</v>
+        <v>-0.041</v>
       </c>
       <c r="V26" s="2" t="inlineStr"/>
       <c r="W26" s="2" t="n">
-        <v>25.63</v>
+        <v>13.62</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>1385752</v>
+        <v>3869975</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>2613156</v>
+        <v>7776210</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>0.53</v>
+        <v>0.5</v>
       </c>
       <c r="AA26" s="2" t="n">
-        <v>441478</v>
+        <v>71207</v>
       </c>
       <c r="AB26" s="2" t="n">
-        <v>38.5179</v>
+        <v>16.530321</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>28.398287</v>
+        <v>12.161287</v>
       </c>
       <c r="AD26" s="2" t="n">
-        <v>14.72</v>
-      </c>
-      <c r="AE26" s="2" t="n">
-        <v>5.517</v>
-      </c>
+        <v>11.73</v>
+      </c>
+      <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="n">
-        <v>12.8</v>
+        <v>12.3</v>
       </c>
       <c r="AG26" s="2" t="n">
-        <v>25.6</v>
+        <v>22.2</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>5.670926</v>
+        <v>1.7787559</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="AJ26" s="2" t="n">
-        <v>2.824</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="AJ26" s="2" t="inlineStr"/>
       <c r="AK26" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/SUNPHARMA/</t>
+          <t>https://www.screener.in/company/FEDERALBNK/</t>
         </is>
       </c>
       <c r="AL26" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:SUNPHARMA</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:FEDERALBNK</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>FEDERALBNK</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>The Federal Bank Limited</t>
+          <t>Tata Steel Limited</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Banks - Regional</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>50.6</v>
+        <v>50</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>23.6</v>
+        <v>17</v>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
@@ -4067,23 +4071,23 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High</t>
+          <t>📈 EMA Bull Stack | 🏆 Near 52W High</t>
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>288.9</v>
+        <v>214.7</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>-0.45</v>
+        <v>2.01</v>
       </c>
       <c r="L27" s="4" t="n">
-        <v>287.49</v>
+        <v>211.55</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>284.75</v>
+        <v>207.68</v>
       </c>
       <c r="N27" s="4" t="n">
-        <v>258.64</v>
+        <v>187.02</v>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
@@ -4092,103 +4096,107 @@
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="Q27" s="4" t="n">
-        <v>95.66</v>
+        <v>95.68000000000001</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>52.42</v>
+        <v>56.32</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.5874</v>
+        <v>0.7458</v>
       </c>
       <c r="T27" s="4" t="n">
-        <v>0.6284</v>
+        <v>1.3924</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>-0.041</v>
+        <v>-0.6466</v>
       </c>
       <c r="V27" s="4" t="inlineStr"/>
       <c r="W27" s="4" t="n">
-        <v>13.62</v>
+        <v>17.08</v>
       </c>
       <c r="X27" s="4" t="n">
-        <v>3869975</v>
+        <v>39110042</v>
       </c>
       <c r="Y27" s="4" t="n">
-        <v>7776210</v>
+        <v>29021368</v>
       </c>
       <c r="Z27" s="4" t="n">
-        <v>0.5</v>
+        <v>1.35</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>71207</v>
+        <v>259439</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>16.530321</v>
+        <v>28.3406</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>12.161287</v>
+        <v>11.064895</v>
       </c>
       <c r="AD27" s="4" t="n">
-        <v>11.73</v>
-      </c>
-      <c r="AE27" s="4" t="inlineStr"/>
+        <v>11.16</v>
+      </c>
+      <c r="AE27" s="4" t="n">
+        <v>89.01600000000001</v>
+      </c>
       <c r="AF27" s="4" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="AG27" s="4" t="n">
-        <v>22.2</v>
+        <v>125.4</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>1.7787559</v>
+        <v>2.7291691</v>
       </c>
       <c r="AI27" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="AJ27" s="4" t="inlineStr"/>
+        <v>186</v>
+      </c>
+      <c r="AJ27" s="4" t="n">
+        <v>0.748</v>
+      </c>
       <c r="AK27" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/FEDERALBNK/</t>
+          <t>https://www.screener.in/company/TATASTEEL/</t>
         </is>
       </c>
       <c r="AL27" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:FEDERALBNK</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:TATASTEEL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HFCL</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Tata Steel Limited</t>
+          <t>HFCL Limited</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Communication Equipment</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
         <v>50</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
@@ -4197,23 +4205,23 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>📈 EMA Bull Stack | 🏆 Near 52W High</t>
+          <t>🔥 Fresh MACD Cross | ✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High</t>
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>214.7</v>
+        <v>173.92</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>2.01</v>
+        <v>7.49</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>211.55</v>
+        <v>141.7</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>207.68</v>
+        <v>117.08</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>187.21</v>
+        <v>87.62</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -4222,87 +4230,89 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>95.68000000000001</v>
+        <v>98.56999999999999</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>56.32</v>
+        <v>80.47</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>0.7458</v>
+        <v>15.3836</v>
       </c>
       <c r="T28" s="2" t="n">
-        <v>1.3924</v>
+        <v>14.6133</v>
       </c>
       <c r="U28" s="2" t="n">
-        <v>-0.6466</v>
-      </c>
-      <c r="V28" s="2" t="inlineStr"/>
+        <v>0.7703</v>
+      </c>
+      <c r="V28" s="2" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="W28" s="2" t="n">
-        <v>17.08</v>
+        <v>58.37</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>39110042</v>
+        <v>79961509</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>29021368</v>
+        <v>90025183</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>1.35</v>
+        <v>0.89</v>
       </c>
       <c r="AA28" s="2" t="n">
-        <v>267534</v>
+        <v>27536</v>
       </c>
       <c r="AB28" s="2" t="n">
-        <v>29.224794</v>
+        <v>486.3243</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>11.410107</v>
+        <v>34.603848</v>
       </c>
       <c r="AD28" s="2" t="n">
-        <v>11.16</v>
+        <v>7.27</v>
       </c>
       <c r="AE28" s="2" t="n">
-        <v>89.01600000000001</v>
+        <v>38.321</v>
       </c>
       <c r="AF28" s="2" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="AG28" s="2" t="n">
-        <v>125.4</v>
-      </c>
+        <v>127.8</v>
+      </c>
+      <c r="AG28" s="2" t="inlineStr"/>
       <c r="AH28" s="2" t="n">
-        <v>2.8143163</v>
+        <v>5.427563</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>186</v>
+        <v>6</v>
       </c>
       <c r="AJ28" s="2" t="n">
-        <v>0.748</v>
+        <v>1.991</v>
       </c>
       <c r="AK28" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/TATASTEEL/</t>
+          <t>https://www.screener.in/company/HFCL/</t>
         </is>
       </c>
       <c r="AL28" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:TATASTEEL</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:HFCL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>HFCL</t>
+          <t>IDEAFORGE</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>HFCL Limited</t>
+          <t>ideaForge Technology Limited</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -4312,17 +4322,17 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Communication Equipment</t>
+          <t>Computer Hardware</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>50</v>
+        <v>49.4</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>10</v>
+        <v>12.4</v>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
@@ -4331,23 +4341,23 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>🔥 Fresh MACD Cross | ✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High</t>
+          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High</t>
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>173.92</v>
+        <v>845.3</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>7.49</v>
+        <v>-1.18</v>
       </c>
       <c r="L29" s="4" t="n">
-        <v>141.7</v>
+        <v>752.75</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>117.08</v>
+        <v>637.05</v>
       </c>
       <c r="N29" s="4" t="n">
-        <v>87.67</v>
+        <v>509.38</v>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
@@ -4360,203 +4370,193 @@
         </is>
       </c>
       <c r="Q29" s="4" t="n">
-        <v>98.56999999999999</v>
+        <v>95.19</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>80.47</v>
+        <v>66.70999999999999</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>15.3836</v>
+        <v>68.745</v>
       </c>
       <c r="T29" s="4" t="n">
-        <v>14.6133</v>
+        <v>73.77549999999999</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>0.7703</v>
-      </c>
-      <c r="V29" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>-5.0305</v>
+      </c>
+      <c r="V29" s="4" t="inlineStr"/>
       <c r="W29" s="4" t="n">
-        <v>58.37</v>
+        <v>39.81</v>
       </c>
       <c r="X29" s="4" t="n">
-        <v>79961509</v>
+        <v>579560</v>
       </c>
       <c r="Y29" s="4" t="n">
-        <v>90025183</v>
+        <v>2450705</v>
       </c>
       <c r="Z29" s="4" t="n">
-        <v>0.89</v>
+        <v>0.24</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>26504</v>
-      </c>
-      <c r="AB29" s="4" t="n">
-        <v>468.1081</v>
-      </c>
+        <v>3666</v>
+      </c>
+      <c r="AB29" s="4" t="inlineStr"/>
       <c r="AC29" s="4" t="n">
-        <v>33.307693</v>
+        <v>30.28674</v>
       </c>
       <c r="AD29" s="4" t="n">
-        <v>7.27</v>
+        <v>-2.82</v>
       </c>
       <c r="AE29" s="4" t="n">
-        <v>38.321</v>
+        <v>13.974</v>
       </c>
       <c r="AF29" s="4" t="n">
-        <v>127.8</v>
+        <v>594.4</v>
       </c>
       <c r="AG29" s="4" t="inlineStr"/>
       <c r="AH29" s="4" t="n">
-        <v>5.224263</v>
+        <v>6.1680183</v>
       </c>
       <c r="AI29" s="4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>1.991</v>
+        <v>2.622</v>
       </c>
       <c r="AK29" s="4" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/HFCL/</t>
+          <t>https://www.screener.in/company/IDEAFORGE/</t>
         </is>
       </c>
       <c r="AL29" s="4" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:HFCL</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:IDEAFORGE</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>IDEAFORGE</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>ideaForge Technology Limited</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Computer Hardware</t>
+          <t>Banks - Regional</t>
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>49.4</v>
+        <v>46.9</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>37</v>
+        <v>25.5</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>12.4</v>
+        <v>21.4</v>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>✅ Supertrend Buy | 📈 EMA Bull Stack | 🏆 Near 52W High</t>
-        </is>
-      </c>
+      <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="n">
-        <v>845.3</v>
+        <v>134.16</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>-1.18</v>
+        <v>0.76</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>752.75</v>
+        <v>132</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>637.05</v>
+        <v>135.46</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>509.74</v>
+        <v>132.94</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✗</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>95.19</v>
+        <v>82.36</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>66.70999999999999</v>
+        <v>52.71</v>
       </c>
       <c r="S30" s="2" t="n">
-        <v>68.745</v>
+        <v>-1.5506</v>
       </c>
       <c r="T30" s="2" t="n">
-        <v>73.77549999999999</v>
+        <v>-2.2398</v>
       </c>
       <c r="U30" s="2" t="n">
-        <v>-5.0305</v>
+        <v>0.6892</v>
       </c>
       <c r="V30" s="2" t="inlineStr"/>
       <c r="W30" s="2" t="n">
-        <v>39.81</v>
+        <v>14.83</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>579560</v>
+        <v>26115218</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>2450705</v>
+        <v>23758342</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>0.24</v>
+        <v>1.1</v>
       </c>
       <c r="AA30" s="2" t="n">
-        <v>3645</v>
-      </c>
-      <c r="AB30" s="2" t="inlineStr"/>
+        <v>118644</v>
+      </c>
+      <c r="AB30" s="2" t="n">
+        <v>6.0193286</v>
+      </c>
       <c r="AC30" s="2" t="n">
-        <v>30.107527</v>
+        <v>5.6615143</v>
       </c>
       <c r="AD30" s="2" t="n">
-        <v>-2.82</v>
-      </c>
-      <c r="AE30" s="2" t="n">
-        <v>13.974</v>
-      </c>
+        <v>15.94</v>
+      </c>
+      <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="n">
-        <v>594.4</v>
-      </c>
-      <c r="AG30" s="2" t="inlineStr"/>
+        <v>-46.7</v>
+      </c>
+      <c r="AG30" s="2" t="n">
+        <v>-9.800000000000001</v>
+      </c>
       <c r="AH30" s="2" t="n">
-        <v>6.131521</v>
+        <v>1.0085589</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ30" s="2" t="n">
-        <v>2.622</v>
-      </c>
+        <v>313</v>
+      </c>
+      <c r="AJ30" s="2" t="inlineStr"/>
       <c r="AK30" s="2" t="inlineStr">
         <is>
-          <t>https://www.screener.in/company/IDEAFORGE/</t>
+          <t>https://www.screener.in/company/CANBK/</t>
         </is>
       </c>
       <c r="AL30" s="2" t="inlineStr">
         <is>
-          <t>https://www.tradingview.com/chart/?symbol=NSE:IDEAFORGE</t>
+          <t>https://www.tradingview.com/chart/?symbol=NSE:CANBK</t>
         </is>
       </c>
     </row>
@@ -4610,10 +4610,10 @@
         <v>2577.09</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>2498.6</v>
+        <v>2498.61</v>
       </c>
       <c r="N31" s="4" t="n">
-        <v>2491.34</v>
+        <v>2492.36</v>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
@@ -4654,13 +4654,13 @@
         <v>0.83</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>256437</v>
+        <v>256111</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>66.741516</v>
+        <v>66.656685</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>53.48437</v>
+        <v>53.416393</v>
       </c>
       <c r="AD31" s="4" t="inlineStr"/>
       <c r="AE31" s="4" t="n">
@@ -4673,7 +4673,7 @@
         <v>-4.6</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>13.090927</v>
+        <v>13.074288</v>
       </c>
       <c r="AI31" s="4" t="n">
         <v>94</v>
@@ -4743,7 +4743,7 @@
         <v>284.4</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>258.62</v>
+        <v>258.35</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -4784,13 +4784,13 @@
         <v>1.81</v>
       </c>
       <c r="AA32" s="2" t="n">
-        <v>343819</v>
+        <v>333881</v>
       </c>
       <c r="AB32" s="2" t="n">
-        <v>8.296904</v>
+        <v>8.057074</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>6.3727264</v>
+        <v>6.097757</v>
       </c>
       <c r="AD32" s="2" t="n">
         <v>12.7</v>
@@ -4805,7 +4805,7 @@
         <v>47.8</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>0.92487305</v>
+        <v>0.8981387</v>
       </c>
       <c r="AI32" s="2" t="n">
         <v>675</v>
@@ -4877,7 +4877,7 @@
         <v>1338.68</v>
       </c>
       <c r="N33" s="4" t="n">
-        <v>1393.43</v>
+        <v>1392.41</v>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
@@ -4918,13 +4918,13 @@
         <v>0.52</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>114869</v>
+        <v>113173</v>
       </c>
       <c r="AB33" s="4" t="n">
-        <v>29.662079</v>
+        <v>29.224031</v>
       </c>
       <c r="AC33" s="4" t="n">
-        <v>22.504675</v>
+        <v>22.172327</v>
       </c>
       <c r="AD33" s="4" t="n">
         <v>11.74</v>
@@ -4939,7 +4939,7 @@
         <v>-54.6</v>
       </c>
       <c r="AH33" s="4" t="n">
-        <v>3.489305</v>
+        <v>3.4377751</v>
       </c>
       <c r="AI33" s="4" t="n">
         <v>92</v>
@@ -5007,7 +5007,7 @@
         <v>1557.69</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1504.69</v>
+        <v>1504.48</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -5048,13 +5048,13 @@
         <v>0.8</v>
       </c>
       <c r="AA34" s="2" t="n">
-        <v>43038</v>
+        <v>42398</v>
       </c>
       <c r="AB34" s="2" t="n">
-        <v>80.18017999999999</v>
+        <v>78.98899</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>47.548252</v>
+        <v>46.841854</v>
       </c>
       <c r="AD34" s="2" t="n">
         <v>13.8</v>
@@ -5069,7 +5069,7 @@
         <v>18.9</v>
       </c>
       <c r="AH34" s="2" t="n">
-        <v>10.603934</v>
+        <v>10.446397</v>
       </c>
       <c r="AI34" s="2" t="n">
         <v>23</v>
@@ -5141,7 +5141,7 @@
         <v>263.8</v>
       </c>
       <c r="N35" s="4" t="n">
-        <v>248.23</v>
+        <v>248.25</v>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
@@ -5182,13 +5182,13 @@
         <v>1.07</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>75511</v>
+        <v>75110</v>
       </c>
       <c r="AB35" s="4" t="n">
-        <v>371.40848</v>
+        <v>369.4366</v>
       </c>
       <c r="AC35" s="4" t="n">
-        <v>98.707115</v>
+        <v>98.18307</v>
       </c>
       <c r="AD35" s="4" t="n">
         <v>14.34</v>
@@ -5203,7 +5203,7 @@
         <v>290.2</v>
       </c>
       <c r="AH35" s="4" t="n">
-        <v>53.240463</v>
+        <v>52.9578</v>
       </c>
       <c r="AI35" s="4" t="n">
         <v>0</v>
@@ -5275,7 +5275,7 @@
         <v>1422.92</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>1445.04</v>
+        <v>1445.31</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -5316,13 +5316,13 @@
         <v>0.3</v>
       </c>
       <c r="AA36" s="2" t="n">
-        <v>150529</v>
+        <v>150916</v>
       </c>
       <c r="AB36" s="2" t="n">
-        <v>61.65069</v>
+        <v>61.80909</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>48.77452</v>
+        <v>48.899837</v>
       </c>
       <c r="AD36" s="2" t="n">
         <v>23.52</v>
@@ -5337,7 +5337,7 @@
         <v>37</v>
       </c>
       <c r="AH36" s="2" t="n">
-        <v>15.759526</v>
+        <v>15.800017</v>
       </c>
       <c r="AI36" s="2" t="n">
         <v>68</v>
@@ -5409,7 +5409,7 @@
         <v>482.46</v>
       </c>
       <c r="N37" s="4" t="n">
-        <v>499.51</v>
+        <v>499.64</v>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
@@ -5450,13 +5450,13 @@
         <v>0.25</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>61553</v>
+        <v>58370</v>
       </c>
       <c r="AB37" s="4" t="n">
-        <v>54.76141</v>
+        <v>51.92946</v>
       </c>
       <c r="AC37" s="4" t="n">
-        <v>41.57027</v>
+        <v>39.420486</v>
       </c>
       <c r="AD37" s="4" t="n">
         <v>17.23</v>
@@ -5471,7 +5471,7 @@
         <v>27.7</v>
       </c>
       <c r="AH37" s="4" t="n">
-        <v>8.903244000000001</v>
+        <v>8.442818000000001</v>
       </c>
       <c r="AI37" s="4" t="n">
         <v>72</v>
@@ -5543,7 +5543,7 @@
         <v>173.31</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>179.44</v>
+        <v>179.1</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -5584,13 +5584,13 @@
         <v>16.67</v>
       </c>
       <c r="AA38" s="2" t="n">
-        <v>11954</v>
+        <v>11514</v>
       </c>
       <c r="AB38" s="2" t="n">
-        <v>19.951498</v>
+        <v>19.21775</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>17.339014</v>
+        <v>16.701345</v>
       </c>
       <c r="AD38" s="2" t="n">
         <v>9.73</v>
@@ -5605,7 +5605,7 @@
         <v>59</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>2.0198083</v>
+        <v>1.9455268</v>
       </c>
       <c r="AI38" s="2" t="n">
         <v>104</v>
@@ -5677,7 +5677,7 @@
         <v>302.77</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>288.89</v>
+        <v>289.15</v>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
@@ -5718,13 +5718,13 @@
         <v>1.03</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>279530</v>
+        <v>270229</v>
       </c>
       <c r="AB39" s="4" t="n">
-        <v>14.9453</v>
+        <v>14.448034</v>
       </c>
       <c r="AC39" s="4" t="n">
-        <v>15.088669</v>
+        <v>14.586634</v>
       </c>
       <c r="AD39" s="4" t="n">
         <v>16.49</v>
@@ -5739,7 +5739,7 @@
         <v>9.6</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>2.7805274</v>
+        <v>2.6880126</v>
       </c>
       <c r="AI39" s="4" t="n">
         <v>408</v>
@@ -5811,7 +5811,7 @@
         <v>1290.17</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>1257.45</v>
+        <v>1256.61</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0.4</v>
       </c>
       <c r="AA40" s="2" t="n">
-        <v>109903</v>
+        <v>108529</v>
       </c>
       <c r="AB40" s="2" t="n">
-        <v>26.195675</v>
+        <v>25.868229</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>20.462101</v>
+        <v>20.206324</v>
       </c>
       <c r="AD40" s="2" t="n">
         <v>11.83</v>
@@ -5873,7 +5873,7 @@
         <v>-86.2</v>
       </c>
       <c r="AH40" s="2" t="n">
-        <v>2.9186106</v>
+        <v>2.882128</v>
       </c>
       <c r="AI40" s="2" t="n">
         <v>61</v>
@@ -5945,7 +5945,7 @@
         <v>413.54</v>
       </c>
       <c r="N41" s="4" t="n">
-        <v>394.12</v>
+        <v>394.03</v>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
@@ -5986,13 +5986,13 @@
         <v>1.03</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>136729</v>
+        <v>134444</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>36.541416</v>
+        <v>35.93083</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>23.972162</v>
+        <v>23.5716</v>
       </c>
       <c r="AD41" s="4" t="n">
         <v>11.34</v>
@@ -6007,7 +6007,7 @@
         <v>-4.6</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>3.6115494</v>
+        <v>3.5512023</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>59</v>
@@ -6075,7 +6075,7 @@
         <v>79.15000000000001</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>79.26000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -6116,13 +6116,13 @@
         <v>1.61</v>
       </c>
       <c r="AA42" s="2" t="n">
-        <v>81325</v>
+        <v>79225</v>
       </c>
       <c r="AB42" s="2" t="n">
-        <v>29.227436</v>
+        <v>28.472925</v>
       </c>
       <c r="AC42" s="2" t="n">
-        <v>12.65</v>
+        <v>12.323438</v>
       </c>
       <c r="AD42" s="2" t="n">
         <v>9.02</v>
@@ -6137,7 +6137,7 @@
         <v>70.59999999999999</v>
       </c>
       <c r="AH42" s="2" t="n">
-        <v>1.9659075</v>
+        <v>1.9151572</v>
       </c>
       <c r="AI42" s="2" t="n">
         <v>237</v>
@@ -6209,7 +6209,7 @@
         <v>434.34</v>
       </c>
       <c r="N43" s="4" t="n">
-        <v>404.13</v>
+        <v>403.86</v>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
@@ -6250,13 +6250,13 @@
         <v>0.59</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>143092</v>
+        <v>141442</v>
       </c>
       <c r="AB43" s="4" t="n">
-        <v>5.5228634</v>
+        <v>5.459177</v>
       </c>
       <c r="AC43" s="4" t="n">
-        <v>6.660777</v>
+        <v>6.583969</v>
       </c>
       <c r="AD43" s="4" t="n">
         <v>20.47</v>
@@ -6271,7 +6271,7 @@
         <v>10.8</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>1.0769273</v>
+        <v>1.0645088</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>337</v>
@@ -6343,7 +6343,7 @@
         <v>1401.53</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>1255.32</v>
+        <v>1252.93</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -6384,13 +6384,13 @@
         <v>0.61</v>
       </c>
       <c r="AA44" s="2" t="n">
-        <v>82388</v>
+        <v>82072</v>
       </c>
       <c r="AB44" s="2" t="n">
-        <v>23.74233</v>
+        <v>23.651136</v>
       </c>
       <c r="AC44" s="2" t="n">
-        <v>16.172697</v>
+        <v>16.110577</v>
       </c>
       <c r="AD44" s="2" t="n">
         <v>9.93</v>
@@ -6405,7 +6405,7 @@
         <v>1.9</v>
       </c>
       <c r="AH44" s="2" t="n">
-        <v>2.1951084</v>
+        <v>2.186677</v>
       </c>
       <c r="AI44" s="2" t="n">
         <v>28</v>
@@ -6477,7 +6477,7 @@
         <v>3417.85</v>
       </c>
       <c r="N45" s="4" t="n">
-        <v>3290.76</v>
+        <v>3281.67</v>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
@@ -6518,13 +6518,13 @@
         <v>0.21</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>132926</v>
+        <v>134207</v>
       </c>
       <c r="AB45" s="4" t="n">
-        <v>12.546894</v>
+        <v>12.667777</v>
       </c>
       <c r="AC45" s="4" t="n">
-        <v>9.570746</v>
+        <v>9.662955999999999</v>
       </c>
       <c r="AD45" s="4" t="n">
         <v>30.41</v>
@@ -6539,7 +6539,7 @@
         <v>126.7</v>
       </c>
       <c r="AH45" s="4" t="n">
-        <v>3.73165</v>
+        <v>3.767603</v>
       </c>
       <c r="AI45" s="4" t="n">
         <v>91</v>
@@ -6608,10 +6608,10 @@
         <v>7701.87</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>7589.88</v>
+        <v>7589.87</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>7246.86</v>
+        <v>7228.7</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -6652,13 +6652,13 @@
         <v>0.75</v>
       </c>
       <c r="AA46" s="2" t="n">
-        <v>26541</v>
+        <v>26856</v>
       </c>
       <c r="AB46" s="2" t="n">
-        <v>149.43407</v>
+        <v>151.21127</v>
       </c>
       <c r="AC46" s="2" t="n">
-        <v>39.591805</v>
+        <v>40.062668</v>
       </c>
       <c r="AD46" s="2" t="n">
         <v>5.58</v>
@@ -6673,7 +6673,7 @@
         <v>11</v>
       </c>
       <c r="AH46" s="2" t="n">
-        <v>6.0578327</v>
+        <v>6.1298776</v>
       </c>
       <c r="AI46" s="2" t="n">
         <v>0</v>
@@ -6745,7 +6745,7 @@
         <v>4225.94</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>3982.04</v>
+        <v>3985.18</v>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
@@ -6786,13 +6786,13 @@
         <v>0.33</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>368567</v>
+        <v>361462</v>
       </c>
       <c r="AB47" s="4" t="n">
-        <v>72.76707500000001</v>
+        <v>71.36427</v>
       </c>
       <c r="AC47" s="4" t="n">
-        <v>48.402096</v>
+        <v>47.468998</v>
       </c>
       <c r="AD47" s="4" t="n">
         <v>37.13</v>
@@ -6807,7 +6807,7 @@
         <v>35.1</v>
       </c>
       <c r="AH47" s="4" t="n">
-        <v>28.778822</v>
+        <v>23.038303</v>
       </c>
       <c r="AI47" s="4" t="n">
         <v>27</v>
@@ -7373,7 +7373,7 @@
         <v>324.82</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>296.89</v>
+        <v>296.83</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -7414,13 +7414,13 @@
         <v>1.01</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>21540</v>
+        <v>21360</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>24.673758</v>
+        <v>24.468084</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>18.331898</v>
+        <v>18.179089</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -7431,7 +7431,7 @@
         <v>367.9</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>1.2857991</v>
+        <v>1.2750812</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>33</v>
@@ -7501,7 +7501,7 @@
         <v>453.89</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>417.78</v>
+        <v>417.31</v>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
@@ -7542,13 +7542,13 @@
         <v>7.74</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>285704</v>
+        <v>282191</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>9.185655000000001</v>
+        <v>9.072716</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>8.106672</v>
+        <v>8.007</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>28.12</v>
@@ -7563,7 +7563,7 @@
         <v>12.9</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>2.3985927</v>
+        <v>2.3691018</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>475</v>
@@ -7635,7 +7635,7 @@
         <v>1641.65</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1490.46</v>
+        <v>1490.49</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -7676,13 +7676,13 @@
         <v>0.66</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>420012</v>
+        <v>415772</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>31.323023</v>
+        <v>31.006872</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>23.50455</v>
+        <v>23.267313</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>15.59</v>
@@ -7697,7 +7697,7 @@
         <v>3.6</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>4.369073</v>
+        <v>4.3249745</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>41</v>
@@ -7769,7 +7769,7 @@
         <v>6510.26</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>6303.62</v>
+        <v>6303.55</v>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
@@ -7810,13 +7810,13 @@
         <v>0.43</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>180280</v>
+        <v>176988</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>70.358475</v>
+        <v>69.07377</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>48.03056</v>
+        <v>47.15355</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>16.19</v>
@@ -7831,7 +7831,7 @@
         <v>13.6</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>11.689433</v>
+        <v>11.47599</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>44</v>
@@ -7903,7 +7903,7 @@
         <v>1189.85</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>1017.63</v>
+        <v>1017.19</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -7944,13 +7944,13 @@
         <v>0.35</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>9965</v>
+        <v>10155</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>88.17967</v>
+        <v>89.86407</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>45.615974</v>
+        <v>46.487324</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>16.94</v>
@@ -7965,7 +7965,7 @@
         <v>69</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>13.810468</v>
+        <v>14.074273</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>0</v>
@@ -8037,7 +8037,7 @@
         <v>8441.25</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>7560.62</v>
+        <v>7561.76</v>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
@@ -8078,13 +8078,13 @@
         <v>0.49</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>145462</v>
+        <v>142684</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>54.63387</v>
+        <v>53.59061</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>39.262745</v>
+        <v>38.51301</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>24.58</v>
@@ -8099,7 +8099,7 @@
         <v>8</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>12.1131735</v>
+        <v>11.881867</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>36</v>
@@ -8171,7 +8171,7 @@
         <v>7830.53</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>7493.93</v>
+        <v>7498.69</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -8212,13 +8212,13 @@
         <v>0.67</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>119047</v>
+        <v>117566</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>61.402405</v>
+        <v>60.638535</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>38.752354</v>
+        <v>38.27026</v>
       </c>
       <c r="AD8" s="2" t="n">
         <v>21.5</v>
@@ -8233,7 +8233,7 @@
         <v>35.6</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>12.554779</v>
+        <v>12.398593</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>24</v>
@@ -8305,7 +8305,7 @@
         <v>4296.48</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>3957.95</v>
+        <v>3950.73</v>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
@@ -8346,13 +8346,13 @@
         <v>0.7</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>153285</v>
+        <v>149282</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>70.789314</v>
+        <v>68.94029</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>47.70262</v>
+        <v>46.456627</v>
       </c>
       <c r="AD9" s="4" t="n">
         <v>16.98</v>
@@ -8367,7 +8367,7 @@
         <v>-21.8</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>18.155107</v>
+        <v>17.680895</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>84</v>
@@ -8439,7 +8439,7 @@
         <v>1249.42</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1171.93</v>
+        <v>1171.38</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -8480,13 +8480,13 @@
         <v>1.14</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>319723</v>
+        <v>311913</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>14.354591</v>
+        <v>14.003944</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>18.041344</v>
+        <v>17.60064</v>
       </c>
       <c r="AD10" s="2" t="n">
         <v>27.26</v>
@@ -8501,7 +8501,7 @@
         <v>991.8</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>3.1956675</v>
+        <v>3.1176054</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>54</v>
@@ -8573,7 +8573,7 @@
         <v>415.21</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>360.58</v>
+        <v>360.33</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -8614,13 +8614,13 @@
         <v>0.16</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>12713</v>
+        <v>12407</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>30.676786</v>
+        <v>29.93991</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>18.210266</v>
+        <v>17.772844</v>
       </c>
       <c r="AD11" s="4" t="n">
         <v>10.66</v>
@@ -8635,7 +8635,7 @@
         <v>-85.59999999999999</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>3.13987</v>
+        <v>22.567343</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>77</v>
@@ -8954,7 +8954,7 @@
         <v>324.82</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>296.89</v>
+        <v>296.83</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -8995,13 +8995,13 @@
         <v>1.01</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>21540</v>
+        <v>21360</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>24.673758</v>
+        <v>24.468084</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>18.331898</v>
+        <v>18.179089</v>
       </c>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
@@ -9012,7 +9012,7 @@
         <v>367.9</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>1.2857991</v>
+        <v>1.2750812</v>
       </c>
       <c r="AI2" s="2" t="n">
         <v>33</v>
@@ -9082,7 +9082,7 @@
         <v>453.89</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>417.78</v>
+        <v>417.31</v>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
@@ -9123,13 +9123,13 @@
         <v>7.74</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>285704</v>
+        <v>282191</v>
       </c>
       <c r="AB3" s="4" t="n">
-        <v>9.185655000000001</v>
+        <v>9.072716</v>
       </c>
       <c r="AC3" s="4" t="n">
-        <v>8.106672</v>
+        <v>8.007</v>
       </c>
       <c r="AD3" s="4" t="n">
         <v>28.12</v>
@@ -9144,7 +9144,7 @@
         <v>12.9</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>2.3985927</v>
+        <v>2.3691018</v>
       </c>
       <c r="AI3" s="4" t="n">
         <v>475</v>
@@ -9216,7 +9216,7 @@
         <v>1641.65</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1490.46</v>
+        <v>1490.49</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -9257,13 +9257,13 @@
         <v>0.66</v>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>420012</v>
+        <v>415772</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>31.323023</v>
+        <v>31.006872</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>23.50455</v>
+        <v>23.267313</v>
       </c>
       <c r="AD4" s="2" t="n">
         <v>15.59</v>
@@ -9278,7 +9278,7 @@
         <v>3.6</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>4.369073</v>
+        <v>4.3249745</v>
       </c>
       <c r="AI4" s="2" t="n">
         <v>41</v>
@@ -9350,7 +9350,7 @@
         <v>6510.26</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>6303.62</v>
+        <v>6303.55</v>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
@@ -9391,13 +9391,13 @@
         <v>0.43</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>180280</v>
+        <v>176988</v>
       </c>
       <c r="AB5" s="4" t="n">
-        <v>70.358475</v>
+        <v>69.07377</v>
       </c>
       <c r="AC5" s="4" t="n">
-        <v>48.03056</v>
+        <v>47.15355</v>
       </c>
       <c r="AD5" s="4" t="n">
         <v>16.19</v>
@@ -9412,7 +9412,7 @@
         <v>13.6</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>11.689433</v>
+        <v>11.47599</v>
       </c>
       <c r="AI5" s="4" t="n">
         <v>44</v>
@@ -9484,7 +9484,7 @@
         <v>1189.85</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>1017.63</v>
+        <v>1017.19</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -9525,13 +9525,13 @@
         <v>0.35</v>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>9965</v>
+        <v>10155</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>88.17967</v>
+        <v>89.86407</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>45.615974</v>
+        <v>46.487324</v>
       </c>
       <c r="AD6" s="2" t="n">
         <v>16.94</v>
@@ -9546,7 +9546,7 @@
         <v>69</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>13.810468</v>
+        <v>14.074273</v>
       </c>
       <c r="AI6" s="2" t="n">
         <v>0</v>
@@ -9618,7 +9618,7 @@
         <v>8441.25</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>7560.62</v>
+        <v>7561.76</v>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
@@ -9659,13 +9659,13 @@
         <v>0.49</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>145462</v>
+        <v>142684</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>54.63387</v>
+        <v>53.59061</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>39.262745</v>
+        <v>38.51301</v>
       </c>
       <c r="AD7" s="4" t="n">
         <v>24.58</v>
@@ -9680,7 +9680,7 @@
         <v>8</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>12.1131735</v>
+        <v>11.881867</v>
       </c>
       <c r="AI7" s="4" t="n">
         <v>36</v>
@@ -9752,7 +9752,7 @@
         <v>7830.53</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>7493.93</v>
+        <v>7498.69</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -9793,13 +9793,13 @@
         <v>0.67</v>
       </c>
       <c r="AA8" s="2" t="n">
-        <v>119047</v>
+        <v>117566</v>
       </c>
       <c r="AB8" s="2" t="n">
-        <v>61.402405</v>
+        <v>60.638535</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>38.752354</v>
+        <v>38.27026</v>
       </c>
       <c r="AD8" s="2" t="n">
         <v>21.5</v>
@@ -9814,7 +9814,7 @@
         <v>35.6</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>12.554779</v>
+        <v>12.398593</v>
       </c>
       <c r="AI8" s="2" t="n">
         <v>24</v>
@@ -9886,7 +9886,7 @@
         <v>4296.48</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>3957.95</v>
+        <v>3950.73</v>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
@@ -9927,13 +9927,13 @@
         <v>0.7</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>153285</v>
+        <v>149282</v>
       </c>
       <c r="AB9" s="4" t="n">
-        <v>70.789314</v>
+        <v>68.94029</v>
       </c>
       <c r="AC9" s="4" t="n">
-        <v>47.70262</v>
+        <v>46.456627</v>
       </c>
       <c r="AD9" s="4" t="n">
         <v>16.98</v>
@@ -9948,7 +9948,7 @@
         <v>-21.8</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>18.155107</v>
+        <v>17.680895</v>
       </c>
       <c r="AI9" s="4" t="n">
         <v>84</v>
@@ -10020,7 +10020,7 @@
         <v>1249.42</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1171.93</v>
+        <v>1171.38</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -10061,13 +10061,13 @@
         <v>1.14</v>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>319723</v>
+        <v>311913</v>
       </c>
       <c r="AB10" s="2" t="n">
-        <v>14.354591</v>
+        <v>14.003944</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>18.041344</v>
+        <v>17.60064</v>
       </c>
       <c r="AD10" s="2" t="n">
         <v>27.26</v>
@@ -10082,7 +10082,7 @@
         <v>991.8</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>3.1956675</v>
+        <v>3.1176054</v>
       </c>
       <c r="AI10" s="2" t="n">
         <v>54</v>
@@ -10154,7 +10154,7 @@
         <v>415.21</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>360.58</v>
+        <v>360.33</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -10195,13 +10195,13 @@
         <v>0.16</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>12713</v>
+        <v>12407</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>30.676786</v>
+        <v>29.93991</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>18.210266</v>
+        <v>17.772844</v>
       </c>
       <c r="AD11" s="4" t="n">
         <v>10.66</v>
@@ -10216,7 +10216,7 @@
         <v>-85.59999999999999</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>3.13987</v>
+        <v>22.567343</v>
       </c>
       <c r="AI11" s="4" t="n">
         <v>77</v>
@@ -10261,7 +10261,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Run Date: 28-May-2026 18:44 IST</t>
+          <t>Run Date: 29-May-2026 18:43 IST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -10365,7 +10365,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>51.1</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14">

</xml_diff>